<commit_message>
Sync local changes: update bot and modules, add new scripts, stop tracking files with DB credentials
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/all_phone.xlsx
+++ b/excel/all_phone.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13548" windowHeight="11580"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13550" windowHeight="11580"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2185" uniqueCount="1131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2217" uniqueCount="1147">
   <si>
     <t>Site</t>
   </si>
@@ -3420,18 +3420,73 @@
   </si>
   <si>
     <t>araya@ncr-rubber.com</t>
+  </si>
+  <si>
+    <t>วิภาวี</t>
+  </si>
+  <si>
+    <t>เจนพาณิชย์ชีพ</t>
+  </si>
+  <si>
+    <t>เต้น</t>
+  </si>
+  <si>
+    <t>WJ</t>
+  </si>
+  <si>
+    <t>wiparwee@ncr-rubber.com</t>
+  </si>
+  <si>
+    <t>เลขานุการกรรมการผู้จัดการ</t>
+  </si>
+  <si>
+    <t>มีนา</t>
+  </si>
+  <si>
+    <t>รัตนมุง</t>
+  </si>
+  <si>
+    <t>MN</t>
+  </si>
+  <si>
+    <t>meena@ncr-rubber.com</t>
+  </si>
+  <si>
+    <t>Sr. International sales executive</t>
+  </si>
+  <si>
+    <t>สมภพ</t>
+  </si>
+  <si>
+    <t>พึ่งฉิม</t>
+  </si>
+  <si>
+    <t>บิ๊ก</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>somphop@ncr-rubber.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -3548,48 +3603,50 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3890,22 +3947,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M251"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <dimension ref="A1:M254"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="3.88671875" customWidth="1"/>
-    <col min="2" max="2" width="7.44140625" customWidth="1"/>
-    <col min="3" max="3" width="8.5546875" customWidth="1"/>
-    <col min="4" max="4" width="16.44140625" customWidth="1"/>
-    <col min="5" max="5" width="15.44140625" customWidth="1"/>
-    <col min="6" max="6" width="10.88671875" customWidth="1"/>
+    <col min="1" max="1" width="3.90625" customWidth="1"/>
+    <col min="2" max="2" width="7.453125" customWidth="1"/>
+    <col min="3" max="3" width="8.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.453125" customWidth="1"/>
+    <col min="5" max="5" width="15.453125" customWidth="1"/>
+    <col min="6" max="6" width="10.90625" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="13.5546875" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" customWidth="1"/>
-    <col min="10" max="10" width="5.88671875" customWidth="1"/>
-    <col min="11" max="11" width="26.109375" customWidth="1"/>
-    <col min="12" max="12" width="31.109375" customWidth="1"/>
-    <col min="13" max="13" width="22.88671875" customWidth="1"/>
+    <col min="8" max="8" width="13.54296875" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" customWidth="1"/>
+    <col min="10" max="10" width="5.90625" customWidth="1"/>
+    <col min="11" max="11" width="26.08984375" customWidth="1"/>
+    <col min="12" max="12" width="31.08984375" customWidth="1"/>
+    <col min="13" max="13" width="22.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -7554,7 +7611,7 @@
         <v>621</v>
       </c>
       <c r="B143" t="s">
-        <v>632</v>
+        <v>624</v>
       </c>
       <c r="D143" t="s">
         <v>625</v>
@@ -7565,26 +7622,26 @@
       <c r="F143" t="s">
         <v>625</v>
       </c>
-      <c r="G143" t="s">
-        <v>633</v>
-      </c>
-      <c r="H143" s="4" t="s">
-        <v>634</v>
-      </c>
-      <c r="I143" t="s">
-        <v>635</v>
-      </c>
-      <c r="J143" t="s">
-        <v>636</v>
-      </c>
-      <c r="K143" s="6" t="s">
-        <v>637</v>
-      </c>
-      <c r="L143" s="7" t="s">
-        <v>638</v>
-      </c>
-    </row>
-    <row r="144" spans="1:12" ht="15.6">
+      <c r="G143" s="29" t="s">
+        <v>1142</v>
+      </c>
+      <c r="H143" s="30" t="s">
+        <v>1143</v>
+      </c>
+      <c r="I143" s="29" t="s">
+        <v>1144</v>
+      </c>
+      <c r="J143" s="29" t="s">
+        <v>1145</v>
+      </c>
+      <c r="K143" s="15" t="s">
+        <v>1146</v>
+      </c>
+      <c r="L143" s="3" t="s">
+        <v>1107</v>
+      </c>
+    </row>
+    <row r="144" spans="1:12">
       <c r="A144" t="s">
         <v>621</v>
       </c>
@@ -7601,22 +7658,25 @@
         <v>625</v>
       </c>
       <c r="G144" t="s">
-        <v>639</v>
-      </c>
-      <c r="H144" s="11" t="s">
-        <v>640</v>
+        <v>633</v>
+      </c>
+      <c r="H144" s="4" t="s">
+        <v>634</v>
       </c>
       <c r="I144" t="s">
-        <v>641</v>
-      </c>
-      <c r="K144" s="8" t="s">
-        <v>642</v>
-      </c>
-      <c r="L144" s="12" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="145" spans="1:12">
+        <v>635</v>
+      </c>
+      <c r="J144" t="s">
+        <v>636</v>
+      </c>
+      <c r="K144" s="6" t="s">
+        <v>637</v>
+      </c>
+      <c r="L144" s="7" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="145" spans="1:12" ht="15.5">
       <c r="A145" t="s">
         <v>621</v>
       </c>
@@ -7633,19 +7693,19 @@
         <v>625</v>
       </c>
       <c r="G145" t="s">
-        <v>644</v>
+        <v>639</v>
       </c>
       <c r="H145" s="11" t="s">
-        <v>645</v>
+        <v>640</v>
       </c>
       <c r="I145" t="s">
-        <v>628</v>
-      </c>
-      <c r="K145" s="6" t="s">
-        <v>646</v>
-      </c>
-      <c r="L145" s="7" t="s">
-        <v>1105</v>
+        <v>641</v>
+      </c>
+      <c r="K145" s="8" t="s">
+        <v>642</v>
+      </c>
+      <c r="L145" s="12" t="s">
+        <v>643</v>
       </c>
     </row>
     <row r="146" spans="1:12">
@@ -7653,7 +7713,7 @@
         <v>621</v>
       </c>
       <c r="B146" t="s">
-        <v>647</v>
+        <v>632</v>
       </c>
       <c r="D146" t="s">
         <v>625</v>
@@ -7665,20 +7725,27 @@
         <v>625</v>
       </c>
       <c r="G146" t="s">
-        <v>648</v>
-      </c>
-      <c r="H146" s="4"/>
-      <c r="K146" s="6"/>
+        <v>644</v>
+      </c>
+      <c r="H146" s="11" t="s">
+        <v>645</v>
+      </c>
+      <c r="I146" t="s">
+        <v>628</v>
+      </c>
+      <c r="K146" s="6" t="s">
+        <v>646</v>
+      </c>
       <c r="L146" s="7" t="s">
-        <v>649</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="147" spans="1:12">
       <c r="A147" t="s">
         <v>621</v>
       </c>
-      <c r="B147">
-        <v>245</v>
+      <c r="B147" t="s">
+        <v>647</v>
       </c>
       <c r="D147" t="s">
         <v>625</v>
@@ -7687,25 +7754,15 @@
         <v>625</v>
       </c>
       <c r="F147" t="s">
-        <v>650</v>
+        <v>625</v>
       </c>
       <c r="G147" t="s">
-        <v>651</v>
-      </c>
-      <c r="H147" s="4" t="s">
-        <v>652</v>
-      </c>
-      <c r="I147" t="s">
-        <v>653</v>
-      </c>
-      <c r="J147" t="s">
-        <v>654</v>
-      </c>
-      <c r="K147" s="6" t="s">
-        <v>655</v>
-      </c>
+        <v>648</v>
+      </c>
+      <c r="H147" s="4"/>
+      <c r="K147" s="6"/>
       <c r="L147" s="7" t="s">
-        <v>656</v>
+        <v>649</v>
       </c>
     </row>
     <row r="148" spans="1:12">
@@ -7713,7 +7770,7 @@
         <v>621</v>
       </c>
       <c r="B148">
-        <v>116</v>
+        <v>245</v>
       </c>
       <c r="D148" t="s">
         <v>625</v>
@@ -7722,22 +7779,25 @@
         <v>625</v>
       </c>
       <c r="F148" t="s">
-        <v>657</v>
+        <v>650</v>
       </c>
       <c r="G148" t="s">
-        <v>658</v>
+        <v>651</v>
       </c>
       <c r="H148" s="4" t="s">
-        <v>659</v>
+        <v>652</v>
       </c>
       <c r="I148" t="s">
-        <v>525</v>
+        <v>653</v>
+      </c>
+      <c r="J148" t="s">
+        <v>654</v>
       </c>
       <c r="K148" s="6" t="s">
-        <v>660</v>
+        <v>655</v>
       </c>
       <c r="L148" s="7" t="s">
-        <v>661</v>
+        <v>656</v>
       </c>
     </row>
     <row r="149" spans="1:12">
@@ -7757,19 +7817,19 @@
         <v>657</v>
       </c>
       <c r="G149" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
       <c r="H149" s="4" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
       <c r="I149" t="s">
-        <v>653</v>
+        <v>525</v>
       </c>
       <c r="K149" s="6" t="s">
-        <v>664</v>
+        <v>660</v>
       </c>
       <c r="L149" s="7" t="s">
-        <v>1106</v>
+        <v>661</v>
       </c>
     </row>
     <row r="150" spans="1:12">
@@ -7777,7 +7837,7 @@
         <v>621</v>
       </c>
       <c r="B150">
-        <v>156</v>
+        <v>116</v>
       </c>
       <c r="D150" t="s">
         <v>625</v>
@@ -7786,30 +7846,30 @@
         <v>625</v>
       </c>
       <c r="F150" t="s">
-        <v>650</v>
+        <v>657</v>
       </c>
       <c r="G150" t="s">
-        <v>523</v>
+        <v>662</v>
       </c>
       <c r="H150" s="4" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
       <c r="I150" t="s">
-        <v>667</v>
+        <v>653</v>
       </c>
       <c r="K150" s="6" t="s">
-        <v>668</v>
+        <v>664</v>
       </c>
       <c r="L150" s="7" t="s">
-        <v>669</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="151" spans="1:12">
       <c r="A151" t="s">
         <v>621</v>
       </c>
-      <c r="B151" t="s">
-        <v>670</v>
+      <c r="B151">
+        <v>156</v>
       </c>
       <c r="D151" t="s">
         <v>625</v>
@@ -7818,51 +7878,51 @@
         <v>625</v>
       </c>
       <c r="F151" t="s">
-        <v>625</v>
+        <v>650</v>
       </c>
       <c r="G151" t="s">
-        <v>671</v>
-      </c>
-      <c r="H151" s="4"/>
+        <v>523</v>
+      </c>
+      <c r="H151" s="4" t="s">
+        <v>666</v>
+      </c>
       <c r="I151" t="s">
-        <v>671</v>
-      </c>
-      <c r="K151" s="6"/>
-      <c r="L151" s="7"/>
+        <v>667</v>
+      </c>
+      <c r="K151" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="L151" s="7" t="s">
+        <v>669</v>
+      </c>
     </row>
     <row r="152" spans="1:12">
       <c r="A152" t="s">
         <v>621</v>
       </c>
       <c r="B152" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="D152" t="s">
-        <v>673</v>
+        <v>625</v>
       </c>
       <c r="E152" t="s">
-        <v>673</v>
+        <v>625</v>
       </c>
       <c r="F152" t="s">
-        <v>674</v>
+        <v>625</v>
       </c>
       <c r="G152" t="s">
-        <v>675</v>
-      </c>
-      <c r="H152" s="4" t="s">
-        <v>676</v>
-      </c>
+        <v>671</v>
+      </c>
+      <c r="H152" s="4"/>
       <c r="I152" t="s">
-        <v>99</v>
-      </c>
-      <c r="K152" s="6" t="s">
-        <v>677</v>
-      </c>
-      <c r="L152" s="7" t="s">
-        <v>678</v>
-      </c>
-    </row>
-    <row r="153" spans="1:12" ht="15.6">
+        <v>671</v>
+      </c>
+      <c r="K152" s="6"/>
+      <c r="L152" s="7"/>
+    </row>
+    <row r="153" spans="1:12">
       <c r="A153" t="s">
         <v>621</v>
       </c>
@@ -7879,27 +7939,27 @@
         <v>674</v>
       </c>
       <c r="G153" t="s">
-        <v>679</v>
+        <v>675</v>
       </c>
       <c r="H153" s="4" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="I153" t="s">
-        <v>681</v>
+        <v>99</v>
       </c>
       <c r="K153" s="6" t="s">
-        <v>682</v>
-      </c>
-      <c r="L153" s="12" t="s">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="154" spans="1:12">
+        <v>677</v>
+      </c>
+      <c r="L153" s="7" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="154" spans="1:12" ht="15.5">
       <c r="A154" t="s">
         <v>621</v>
       </c>
       <c r="B154" t="s">
-        <v>684</v>
+        <v>672</v>
       </c>
       <c r="D154" t="s">
         <v>673</v>
@@ -7911,22 +7971,19 @@
         <v>674</v>
       </c>
       <c r="G154" t="s">
-        <v>685</v>
+        <v>679</v>
       </c>
       <c r="H154" s="4" t="s">
-        <v>686</v>
+        <v>680</v>
       </c>
       <c r="I154" t="s">
-        <v>687</v>
-      </c>
-      <c r="J154" t="s">
-        <v>688</v>
+        <v>681</v>
       </c>
       <c r="K154" s="6" t="s">
-        <v>689</v>
-      </c>
-      <c r="L154" s="7" t="s">
-        <v>1107</v>
+        <v>682</v>
+      </c>
+      <c r="L154" s="12" t="s">
+        <v>683</v>
       </c>
     </row>
     <row r="155" spans="1:12">
@@ -7934,7 +7991,7 @@
         <v>621</v>
       </c>
       <c r="B155" t="s">
-        <v>690</v>
+        <v>684</v>
       </c>
       <c r="D155" t="s">
         <v>673</v>
@@ -7946,25 +8003,25 @@
         <v>674</v>
       </c>
       <c r="G155" t="s">
-        <v>691</v>
+        <v>685</v>
       </c>
       <c r="H155" s="4" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
       <c r="I155" t="s">
-        <v>693</v>
+        <v>687</v>
       </c>
       <c r="J155" t="s">
-        <v>694</v>
-      </c>
-      <c r="K155" s="15" t="s">
-        <v>695</v>
+        <v>688</v>
+      </c>
+      <c r="K155" s="6" t="s">
+        <v>689</v>
       </c>
       <c r="L155" s="7" t="s">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="156" spans="1:12" ht="15.6">
+        <v>1107</v>
+      </c>
+    </row>
+    <row r="156" spans="1:12">
       <c r="A156" t="s">
         <v>621</v>
       </c>
@@ -7981,27 +8038,30 @@
         <v>674</v>
       </c>
       <c r="G156" t="s">
-        <v>696</v>
+        <v>691</v>
       </c>
       <c r="H156" s="4" t="s">
-        <v>697</v>
+        <v>692</v>
       </c>
       <c r="I156" t="s">
-        <v>698</v>
-      </c>
-      <c r="K156" s="6" t="s">
-        <v>699</v>
-      </c>
-      <c r="L156" s="12" t="s">
+        <v>693</v>
+      </c>
+      <c r="J156" t="s">
+        <v>694</v>
+      </c>
+      <c r="K156" s="15" t="s">
+        <v>695</v>
+      </c>
+      <c r="L156" s="7" t="s">
         <v>683</v>
       </c>
     </row>
-    <row r="157" spans="1:12">
+    <row r="157" spans="1:12" ht="15.5">
       <c r="A157" t="s">
         <v>621</v>
       </c>
       <c r="B157" t="s">
-        <v>700</v>
+        <v>690</v>
       </c>
       <c r="D157" t="s">
         <v>673</v>
@@ -8013,22 +8073,22 @@
         <v>674</v>
       </c>
       <c r="G157" t="s">
-        <v>701</v>
+        <v>696</v>
       </c>
       <c r="H157" s="4" t="s">
-        <v>702</v>
+        <v>697</v>
       </c>
       <c r="I157" t="s">
-        <v>703</v>
-      </c>
-      <c r="K157" s="15" t="s">
-        <v>704</v>
-      </c>
-      <c r="L157" s="7" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="158" spans="1:12" ht="15.6">
+        <v>698</v>
+      </c>
+      <c r="K157" s="6" t="s">
+        <v>699</v>
+      </c>
+      <c r="L157" s="12" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="158" spans="1:12">
       <c r="A158" t="s">
         <v>621</v>
       </c>
@@ -8045,27 +8105,27 @@
         <v>674</v>
       </c>
       <c r="G158" t="s">
-        <v>705</v>
-      </c>
-      <c r="H158" s="11" t="s">
-        <v>706</v>
+        <v>701</v>
+      </c>
+      <c r="H158" s="4" t="s">
+        <v>702</v>
       </c>
       <c r="I158" t="s">
-        <v>221</v>
-      </c>
-      <c r="K158" s="6" t="s">
-        <v>707</v>
-      </c>
-      <c r="L158" s="13" t="s">
-        <v>661</v>
-      </c>
-    </row>
-    <row r="159" spans="1:12" ht="15.6">
+        <v>703</v>
+      </c>
+      <c r="K158" s="15" t="s">
+        <v>704</v>
+      </c>
+      <c r="L158" s="7" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="159" spans="1:12" ht="15.5">
       <c r="A159" t="s">
         <v>621</v>
       </c>
       <c r="B159" t="s">
-        <v>708</v>
+        <v>700</v>
       </c>
       <c r="D159" t="s">
         <v>673</v>
@@ -8077,22 +8137,22 @@
         <v>674</v>
       </c>
       <c r="G159" t="s">
-        <v>709</v>
-      </c>
-      <c r="H159" s="4" t="s">
-        <v>710</v>
+        <v>705</v>
+      </c>
+      <c r="H159" s="11" t="s">
+        <v>706</v>
       </c>
       <c r="I159" t="s">
-        <v>711</v>
-      </c>
-      <c r="K159" s="16" t="s">
-        <v>712</v>
-      </c>
-      <c r="L159" s="12" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="160" spans="1:12" ht="15.6">
+        <v>221</v>
+      </c>
+      <c r="K159" s="6" t="s">
+        <v>707</v>
+      </c>
+      <c r="L159" s="13" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="160" spans="1:12" ht="15.5">
       <c r="A160" t="s">
         <v>621</v>
       </c>
@@ -8109,54 +8169,54 @@
         <v>674</v>
       </c>
       <c r="G160" t="s">
+        <v>709</v>
+      </c>
+      <c r="H160" s="4" t="s">
+        <v>710</v>
+      </c>
+      <c r="I160" t="s">
+        <v>711</v>
+      </c>
+      <c r="K160" s="16" t="s">
+        <v>712</v>
+      </c>
+      <c r="L160" s="12" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="161" spans="1:13" ht="15.5">
+      <c r="A161" t="s">
+        <v>621</v>
+      </c>
+      <c r="B161" t="s">
+        <v>708</v>
+      </c>
+      <c r="D161" t="s">
+        <v>673</v>
+      </c>
+      <c r="E161" t="s">
+        <v>673</v>
+      </c>
+      <c r="F161" t="s">
+        <v>674</v>
+      </c>
+      <c r="G161" t="s">
         <v>713</v>
       </c>
-      <c r="H160" s="4" t="s">
+      <c r="H161" s="4" t="s">
         <v>714</v>
       </c>
-      <c r="I160" t="s">
+      <c r="I161" t="s">
         <v>715</v>
       </c>
-      <c r="J160" t="s">
+      <c r="J161" t="s">
         <v>716</v>
       </c>
-      <c r="K160" s="6" t="s">
+      <c r="K161" s="6" t="s">
         <v>717</v>
       </c>
-      <c r="L160" s="12" t="s">
+      <c r="L161" s="12" t="s">
         <v>683</v>
-      </c>
-    </row>
-    <row r="161" spans="1:13">
-      <c r="A161" t="s">
-        <v>621</v>
-      </c>
-      <c r="B161" t="s">
-        <v>718</v>
-      </c>
-      <c r="D161" t="s">
-        <v>719</v>
-      </c>
-      <c r="E161" t="s">
-        <v>719</v>
-      </c>
-      <c r="F161" t="s">
-        <v>720</v>
-      </c>
-      <c r="G161" t="s">
-        <v>721</v>
-      </c>
-      <c r="H161" s="4" t="s">
-        <v>722</v>
-      </c>
-      <c r="I161" t="s">
-        <v>723</v>
-      </c>
-      <c r="K161" s="6" t="s">
-        <v>724</v>
-      </c>
-      <c r="L161" s="7" t="s">
-        <v>725</v>
       </c>
     </row>
     <row r="162" spans="1:13">
@@ -8176,19 +8236,19 @@
         <v>720</v>
       </c>
       <c r="G162" t="s">
-        <v>726</v>
+        <v>721</v>
       </c>
       <c r="H162" s="4" t="s">
-        <v>727</v>
+        <v>722</v>
       </c>
       <c r="I162" t="s">
-        <v>728</v>
+        <v>723</v>
       </c>
       <c r="K162" s="6" t="s">
-        <v>729</v>
+        <v>724</v>
       </c>
       <c r="L162" s="7" t="s">
-        <v>1108</v>
+        <v>725</v>
       </c>
     </row>
     <row r="163" spans="1:13">
@@ -8196,7 +8256,7 @@
         <v>621</v>
       </c>
       <c r="B163" t="s">
-        <v>730</v>
+        <v>718</v>
       </c>
       <c r="D163" t="s">
         <v>719</v>
@@ -8208,25 +8268,22 @@
         <v>720</v>
       </c>
       <c r="G163" t="s">
-        <v>731</v>
+        <v>726</v>
       </c>
       <c r="H163" s="4" t="s">
-        <v>732</v>
+        <v>727</v>
       </c>
       <c r="I163" t="s">
-        <v>733</v>
-      </c>
-      <c r="J163" t="s">
-        <v>734</v>
+        <v>728</v>
       </c>
       <c r="K163" s="6" t="s">
-        <v>735</v>
+        <v>729</v>
       </c>
       <c r="L163" s="7" t="s">
-        <v>736</v>
-      </c>
-    </row>
-    <row r="164" spans="1:13" ht="15.6">
+        <v>1108</v>
+      </c>
+    </row>
+    <row r="164" spans="1:13">
       <c r="A164" t="s">
         <v>621</v>
       </c>
@@ -8243,27 +8300,30 @@
         <v>720</v>
       </c>
       <c r="G164" t="s">
-        <v>737</v>
+        <v>731</v>
       </c>
       <c r="H164" s="4" t="s">
-        <v>738</v>
+        <v>732</v>
       </c>
       <c r="I164" t="s">
-        <v>739</v>
+        <v>733</v>
+      </c>
+      <c r="J164" t="s">
+        <v>734</v>
       </c>
       <c r="K164" s="6" t="s">
-        <v>740</v>
-      </c>
-      <c r="L164" s="12" t="s">
-        <v>741</v>
-      </c>
-    </row>
-    <row r="165" spans="1:13">
+        <v>735</v>
+      </c>
+      <c r="L164" s="7" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="165" spans="1:13" ht="15.5">
       <c r="A165" t="s">
         <v>621</v>
       </c>
       <c r="B165" t="s">
-        <v>742</v>
+        <v>730</v>
       </c>
       <c r="D165" t="s">
         <v>719</v>
@@ -8275,22 +8335,19 @@
         <v>720</v>
       </c>
       <c r="G165" t="s">
-        <v>743</v>
+        <v>737</v>
       </c>
       <c r="H165" s="4" t="s">
-        <v>744</v>
+        <v>738</v>
       </c>
       <c r="I165" t="s">
-        <v>745</v>
-      </c>
-      <c r="J165" t="s">
-        <v>746</v>
-      </c>
-      <c r="K165" s="15" t="s">
-        <v>747</v>
-      </c>
-      <c r="L165" s="7" t="s">
-        <v>748</v>
+        <v>739</v>
+      </c>
+      <c r="K165" s="6" t="s">
+        <v>740</v>
+      </c>
+      <c r="L165" s="12" t="s">
+        <v>741</v>
       </c>
     </row>
     <row r="166" spans="1:13">
@@ -8298,7 +8355,7 @@
         <v>621</v>
       </c>
       <c r="B166" t="s">
-        <v>749</v>
+        <v>742</v>
       </c>
       <c r="D166" t="s">
         <v>719</v>
@@ -8310,27 +8367,30 @@
         <v>720</v>
       </c>
       <c r="G166" t="s">
-        <v>750</v>
+        <v>743</v>
       </c>
       <c r="H166" s="4" t="s">
-        <v>751</v>
+        <v>744</v>
       </c>
       <c r="I166" t="s">
-        <v>752</v>
-      </c>
-      <c r="K166" s="6" t="s">
-        <v>753</v>
+        <v>745</v>
+      </c>
+      <c r="J166" t="s">
+        <v>746</v>
+      </c>
+      <c r="K166" s="15" t="s">
+        <v>747</v>
       </c>
       <c r="L166" s="7" t="s">
-        <v>741</v>
-      </c>
-    </row>
-    <row r="167" spans="1:13" ht="15.6">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="167" spans="1:13">
       <c r="A167" t="s">
         <v>621</v>
       </c>
       <c r="B167" t="s">
-        <v>43</v>
+        <v>749</v>
       </c>
       <c r="D167" t="s">
         <v>719</v>
@@ -8339,33 +8399,30 @@
         <v>719</v>
       </c>
       <c r="F167" t="s">
-        <v>293</v>
+        <v>720</v>
       </c>
       <c r="G167" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="H167" s="4" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="I167" t="s">
-        <v>756</v>
-      </c>
-      <c r="J167" t="s">
-        <v>757</v>
-      </c>
-      <c r="K167" s="8" t="s">
-        <v>758</v>
-      </c>
-      <c r="L167" s="13" t="s">
-        <v>759</v>
-      </c>
-    </row>
-    <row r="168" spans="1:13">
+        <v>752</v>
+      </c>
+      <c r="K167" s="6" t="s">
+        <v>753</v>
+      </c>
+      <c r="L167" s="7" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="168" spans="1:13" ht="15.5">
       <c r="A168" t="s">
         <v>621</v>
       </c>
       <c r="B168" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D168" t="s">
         <v>719</v>
@@ -8377,30 +8434,30 @@
         <v>293</v>
       </c>
       <c r="G168" t="s">
-        <v>760</v>
+        <v>754</v>
       </c>
       <c r="H168" s="4" t="s">
-        <v>761</v>
+        <v>755</v>
       </c>
       <c r="I168" t="s">
-        <v>762</v>
+        <v>756</v>
       </c>
       <c r="J168" t="s">
-        <v>763</v>
-      </c>
-      <c r="K168" s="14" t="s">
-        <v>1109</v>
-      </c>
-      <c r="L168" s="7" t="s">
-        <v>764</v>
-      </c>
-    </row>
-    <row r="169" spans="1:13" ht="15.6">
+        <v>757</v>
+      </c>
+      <c r="K168" s="8" t="s">
+        <v>758</v>
+      </c>
+      <c r="L168" s="13" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="169" spans="1:13">
       <c r="A169" t="s">
         <v>621</v>
       </c>
       <c r="B169" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D169" t="s">
         <v>719</v>
@@ -8412,30 +8469,30 @@
         <v>293</v>
       </c>
       <c r="G169" t="s">
-        <v>765</v>
+        <v>760</v>
       </c>
       <c r="H169" s="4" t="s">
-        <v>766</v>
+        <v>761</v>
       </c>
       <c r="I169" t="s">
-        <v>767</v>
-      </c>
-      <c r="K169" s="8" t="s">
-        <v>768</v>
-      </c>
-      <c r="L169" s="13" t="s">
-        <v>665</v>
-      </c>
-      <c r="M169" t="s">
-        <v>769</v>
-      </c>
-    </row>
-    <row r="170" spans="1:13">
+        <v>762</v>
+      </c>
+      <c r="J169" t="s">
+        <v>763</v>
+      </c>
+      <c r="K169" s="14" t="s">
+        <v>1109</v>
+      </c>
+      <c r="L169" s="7" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="170" spans="1:13" ht="15.5">
       <c r="A170" t="s">
         <v>621</v>
       </c>
       <c r="B170" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D170" t="s">
         <v>719</v>
@@ -8447,22 +8504,25 @@
         <v>293</v>
       </c>
       <c r="G170" t="s">
-        <v>770</v>
+        <v>765</v>
       </c>
       <c r="H170" s="4" t="s">
-        <v>771</v>
+        <v>766</v>
       </c>
       <c r="I170" t="s">
-        <v>772</v>
-      </c>
-      <c r="K170" s="6" t="s">
-        <v>773</v>
-      </c>
-      <c r="L170" s="7" t="s">
-        <v>725</v>
-      </c>
-    </row>
-    <row r="171" spans="1:13" ht="15.6">
+        <v>767</v>
+      </c>
+      <c r="K170" s="8" t="s">
+        <v>768</v>
+      </c>
+      <c r="L170" s="13" t="s">
+        <v>665</v>
+      </c>
+      <c r="M170" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="171" spans="1:13">
       <c r="A171" t="s">
         <v>621</v>
       </c>
@@ -8479,27 +8539,27 @@
         <v>293</v>
       </c>
       <c r="G171" t="s">
-        <v>774</v>
-      </c>
-      <c r="H171" s="11" t="s">
-        <v>775</v>
+        <v>770</v>
+      </c>
+      <c r="H171" s="4" t="s">
+        <v>771</v>
       </c>
       <c r="I171" t="s">
-        <v>776</v>
-      </c>
-      <c r="K171" s="8" t="s">
-        <v>777</v>
-      </c>
-      <c r="L171" s="12" t="s">
+        <v>772</v>
+      </c>
+      <c r="K171" s="6" t="s">
+        <v>773</v>
+      </c>
+      <c r="L171" s="7" t="s">
         <v>725</v>
       </c>
     </row>
-    <row r="172" spans="1:13">
+    <row r="172" spans="1:13" ht="15.5">
       <c r="A172" t="s">
         <v>621</v>
       </c>
       <c r="B172" t="s">
-        <v>778</v>
+        <v>49</v>
       </c>
       <c r="D172" t="s">
         <v>719</v>
@@ -8511,25 +8571,19 @@
         <v>293</v>
       </c>
       <c r="G172" t="s">
-        <v>779</v>
-      </c>
-      <c r="H172" s="4" t="s">
-        <v>780</v>
+        <v>774</v>
+      </c>
+      <c r="H172" s="11" t="s">
+        <v>775</v>
       </c>
       <c r="I172" t="s">
-        <v>781</v>
-      </c>
-      <c r="J172" t="s">
-        <v>782</v>
-      </c>
-      <c r="K172" s="15" t="s">
-        <v>783</v>
-      </c>
-      <c r="L172" s="7" t="s">
-        <v>784</v>
-      </c>
-      <c r="M172" t="s">
-        <v>785</v>
+        <v>776</v>
+      </c>
+      <c r="K172" s="8" t="s">
+        <v>777</v>
+      </c>
+      <c r="L172" s="12" t="s">
+        <v>725</v>
       </c>
     </row>
     <row r="173" spans="1:13">
@@ -8537,7 +8591,7 @@
         <v>621</v>
       </c>
       <c r="B173" t="s">
-        <v>786</v>
+        <v>778</v>
       </c>
       <c r="D173" t="s">
         <v>719</v>
@@ -8549,19 +8603,25 @@
         <v>293</v>
       </c>
       <c r="G173" t="s">
-        <v>787</v>
+        <v>779</v>
       </c>
       <c r="H173" s="4" t="s">
-        <v>788</v>
+        <v>780</v>
       </c>
       <c r="I173" t="s">
-        <v>789</v>
-      </c>
-      <c r="K173" s="6" t="s">
-        <v>790</v>
+        <v>781</v>
+      </c>
+      <c r="J173" t="s">
+        <v>782</v>
+      </c>
+      <c r="K173" s="15" t="s">
+        <v>783</v>
       </c>
       <c r="L173" s="7" t="s">
-        <v>791</v>
+        <v>784</v>
+      </c>
+      <c r="M173" t="s">
+        <v>785</v>
       </c>
     </row>
     <row r="174" spans="1:13">
@@ -8569,37 +8629,34 @@
         <v>621</v>
       </c>
       <c r="B174" t="s">
-        <v>792</v>
+        <v>786</v>
       </c>
       <c r="D174" t="s">
-        <v>793</v>
+        <v>719</v>
       </c>
       <c r="E174" t="s">
-        <v>793</v>
+        <v>719</v>
       </c>
       <c r="F174" t="s">
-        <v>793</v>
+        <v>293</v>
       </c>
       <c r="G174" t="s">
-        <v>794</v>
+        <v>787</v>
       </c>
       <c r="H174" s="4" t="s">
-        <v>795</v>
+        <v>788</v>
       </c>
       <c r="I174" t="s">
-        <v>796</v>
-      </c>
-      <c r="J174" t="s">
-        <v>797</v>
+        <v>789</v>
       </c>
       <c r="K174" s="6" t="s">
-        <v>798</v>
+        <v>790</v>
       </c>
       <c r="L174" s="7" t="s">
-        <v>799</v>
-      </c>
-    </row>
-    <row r="175" spans="1:13" ht="15.6">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="175" spans="1:13">
       <c r="A175" t="s">
         <v>621</v>
       </c>
@@ -8616,19 +8673,22 @@
         <v>793</v>
       </c>
       <c r="G175" t="s">
-        <v>454</v>
+        <v>794</v>
       </c>
       <c r="H175" s="4" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="I175" t="s">
-        <v>801</v>
+        <v>796</v>
+      </c>
+      <c r="J175" t="s">
+        <v>797</v>
       </c>
       <c r="K175" s="6" t="s">
-        <v>802</v>
-      </c>
-      <c r="L175" s="12" t="s">
-        <v>803</v>
+        <v>798</v>
+      </c>
+      <c r="L175" s="7" t="s">
+        <v>799</v>
       </c>
     </row>
     <row r="176" spans="1:13">
@@ -8636,7 +8696,7 @@
         <v>621</v>
       </c>
       <c r="B176" t="s">
-        <v>804</v>
+        <v>792</v>
       </c>
       <c r="D176" t="s">
         <v>793</v>
@@ -8647,31 +8707,31 @@
       <c r="F176" t="s">
         <v>793</v>
       </c>
-      <c r="G176" t="s">
-        <v>805</v>
-      </c>
-      <c r="H176" s="4" t="s">
-        <v>806</v>
-      </c>
-      <c r="I176" t="s">
-        <v>807</v>
-      </c>
-      <c r="J176" t="s">
-        <v>808</v>
-      </c>
-      <c r="K176" s="6" t="s">
-        <v>809</v>
-      </c>
-      <c r="L176" s="7" t="s">
-        <v>810</v>
-      </c>
-    </row>
-    <row r="177" spans="1:12">
+      <c r="G176" s="29" t="s">
+        <v>1137</v>
+      </c>
+      <c r="H176" s="30" t="s">
+        <v>1138</v>
+      </c>
+      <c r="I176" s="29" t="s">
+        <v>256</v>
+      </c>
+      <c r="J176" s="29" t="s">
+        <v>1139</v>
+      </c>
+      <c r="K176" s="15" t="s">
+        <v>1140</v>
+      </c>
+      <c r="L176" s="29" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="177" spans="1:12" ht="15.5">
       <c r="A177" t="s">
         <v>621</v>
       </c>
-      <c r="B177">
-        <v>149</v>
+      <c r="B177" t="s">
+        <v>792</v>
       </c>
       <c r="D177" t="s">
         <v>793</v>
@@ -8683,22 +8743,19 @@
         <v>793</v>
       </c>
       <c r="G177" t="s">
-        <v>811</v>
+        <v>454</v>
       </c>
       <c r="H177" s="4" t="s">
-        <v>812</v>
+        <v>800</v>
       </c>
       <c r="I177" t="s">
-        <v>813</v>
-      </c>
-      <c r="J177" t="s">
-        <v>814</v>
+        <v>801</v>
       </c>
       <c r="K177" s="6" t="s">
-        <v>815</v>
-      </c>
-      <c r="L177" s="7" t="s">
-        <v>816</v>
+        <v>802</v>
+      </c>
+      <c r="L177" s="12" t="s">
+        <v>803</v>
       </c>
     </row>
     <row r="178" spans="1:12">
@@ -8706,7 +8763,7 @@
         <v>621</v>
       </c>
       <c r="B178" t="s">
-        <v>817</v>
+        <v>804</v>
       </c>
       <c r="D178" t="s">
         <v>793</v>
@@ -8718,22 +8775,22 @@
         <v>793</v>
       </c>
       <c r="G178" t="s">
-        <v>818</v>
+        <v>805</v>
       </c>
       <c r="H178" s="4" t="s">
-        <v>819</v>
+        <v>806</v>
       </c>
       <c r="I178" t="s">
-        <v>820</v>
+        <v>807</v>
       </c>
       <c r="J178" t="s">
-        <v>821</v>
+        <v>808</v>
       </c>
       <c r="K178" s="6" t="s">
-        <v>822</v>
+        <v>809</v>
       </c>
       <c r="L178" s="7" t="s">
-        <v>799</v>
+        <v>810</v>
       </c>
     </row>
     <row r="179" spans="1:12">
@@ -8741,7 +8798,7 @@
         <v>621</v>
       </c>
       <c r="B179">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D179" t="s">
         <v>793</v>
@@ -8753,30 +8810,30 @@
         <v>793</v>
       </c>
       <c r="G179" t="s">
-        <v>823</v>
+        <v>811</v>
       </c>
       <c r="H179" s="4" t="s">
-        <v>824</v>
+        <v>812</v>
       </c>
       <c r="I179" t="s">
-        <v>825</v>
+        <v>813</v>
       </c>
       <c r="J179" t="s">
-        <v>826</v>
+        <v>814</v>
       </c>
       <c r="K179" s="6" t="s">
-        <v>827</v>
+        <v>815</v>
       </c>
       <c r="L179" s="7" t="s">
-        <v>828</v>
+        <v>816</v>
       </c>
     </row>
     <row r="180" spans="1:12">
       <c r="A180" t="s">
         <v>621</v>
       </c>
-      <c r="B180">
-        <v>146</v>
+      <c r="B180" t="s">
+        <v>817</v>
       </c>
       <c r="D180" t="s">
         <v>793</v>
@@ -8788,22 +8845,22 @@
         <v>793</v>
       </c>
       <c r="G180" t="s">
-        <v>829</v>
+        <v>818</v>
       </c>
       <c r="H180" s="4" t="s">
-        <v>830</v>
+        <v>819</v>
       </c>
       <c r="I180" t="s">
-        <v>831</v>
+        <v>820</v>
       </c>
       <c r="J180" t="s">
-        <v>832</v>
+        <v>821</v>
       </c>
       <c r="K180" s="6" t="s">
-        <v>833</v>
+        <v>822</v>
       </c>
       <c r="L180" s="7" t="s">
-        <v>834</v>
+        <v>799</v>
       </c>
     </row>
     <row r="181" spans="1:12">
@@ -8823,27 +8880,30 @@
         <v>793</v>
       </c>
       <c r="G181" t="s">
-        <v>493</v>
+        <v>823</v>
       </c>
       <c r="H181" s="4" t="s">
-        <v>835</v>
+        <v>824</v>
       </c>
       <c r="I181" t="s">
-        <v>836</v>
+        <v>825</v>
+      </c>
+      <c r="J181" t="s">
+        <v>826</v>
       </c>
       <c r="K181" s="6" t="s">
-        <v>837</v>
+        <v>827</v>
       </c>
       <c r="L181" s="7" t="s">
-        <v>838</v>
-      </c>
-    </row>
-    <row r="182" spans="1:12" ht="15.6">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="182" spans="1:12">
       <c r="A182" t="s">
         <v>621</v>
       </c>
       <c r="B182">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D182" t="s">
         <v>793</v>
@@ -8855,115 +8915,118 @@
         <v>793</v>
       </c>
       <c r="G182" t="s">
+        <v>829</v>
+      </c>
+      <c r="H182" s="4" t="s">
+        <v>830</v>
+      </c>
+      <c r="I182" t="s">
+        <v>831</v>
+      </c>
+      <c r="J182" t="s">
+        <v>832</v>
+      </c>
+      <c r="K182" s="6" t="s">
+        <v>833</v>
+      </c>
+      <c r="L182" s="7" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="183" spans="1:12">
+      <c r="A183" t="s">
+        <v>621</v>
+      </c>
+      <c r="B183">
+        <v>148</v>
+      </c>
+      <c r="D183" t="s">
+        <v>793</v>
+      </c>
+      <c r="E183" t="s">
+        <v>793</v>
+      </c>
+      <c r="F183" t="s">
+        <v>793</v>
+      </c>
+      <c r="G183" t="s">
+        <v>493</v>
+      </c>
+      <c r="H183" s="4" t="s">
+        <v>835</v>
+      </c>
+      <c r="I183" t="s">
+        <v>836</v>
+      </c>
+      <c r="K183" s="6" t="s">
+        <v>837</v>
+      </c>
+      <c r="L183" s="7" t="s">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="184" spans="1:12" ht="15.5">
+      <c r="A184" t="s">
+        <v>621</v>
+      </c>
+      <c r="B184">
+        <v>143</v>
+      </c>
+      <c r="D184" t="s">
+        <v>793</v>
+      </c>
+      <c r="E184" t="s">
+        <v>793</v>
+      </c>
+      <c r="F184" t="s">
+        <v>793</v>
+      </c>
+      <c r="G184" t="s">
         <v>658</v>
       </c>
-      <c r="H182" s="4" t="s">
+      <c r="H184" s="4" t="s">
         <v>659</v>
       </c>
-      <c r="I182" t="s">
+      <c r="I184" t="s">
         <v>839</v>
       </c>
-      <c r="K182" s="6" t="s">
+      <c r="K184" s="6" t="s">
         <v>660</v>
       </c>
-      <c r="L182" s="13" t="s">
+      <c r="L184" s="13" t="s">
         <v>838</v>
       </c>
     </row>
-    <row r="183" spans="1:12" s="23" customFormat="1">
-      <c r="A183" s="23" t="s">
-        <v>621</v>
-      </c>
-      <c r="B183" s="23">
+    <row r="185" spans="1:12" s="23" customFormat="1">
+      <c r="A185" s="23" t="s">
+        <v>621</v>
+      </c>
+      <c r="B185" s="23">
         <v>147</v>
       </c>
-      <c r="D183" s="23" t="s">
+      <c r="D185" s="23" t="s">
         <v>1012</v>
       </c>
-      <c r="E183" s="23" t="s">
+      <c r="E185" s="23" t="s">
         <v>1012</v>
       </c>
-      <c r="F183" s="23" t="s">
+      <c r="F185" s="23" t="s">
         <v>1012</v>
       </c>
-      <c r="G183" s="23" t="s">
+      <c r="G185" s="23" t="s">
         <v>841</v>
       </c>
-      <c r="H183" s="25" t="s">
+      <c r="H185" s="25" t="s">
         <v>761</v>
       </c>
-      <c r="I183" s="25" t="s">
+      <c r="I185" s="25" t="s">
         <v>1126</v>
       </c>
-      <c r="K183" s="28" t="s">
+      <c r="K185" s="28" t="s">
         <v>842</v>
       </c>
-      <c r="L183" s="23" t="s">
+      <c r="L185" s="23" t="s">
         <v>485</v>
-      </c>
-    </row>
-    <row r="184" spans="1:12">
-      <c r="A184" t="s">
-        <v>621</v>
-      </c>
-      <c r="B184" t="s">
-        <v>843</v>
-      </c>
-      <c r="D184" t="s">
-        <v>840</v>
-      </c>
-      <c r="E184" t="s">
-        <v>840</v>
-      </c>
-      <c r="F184" t="s">
-        <v>840</v>
-      </c>
-      <c r="G184" t="s">
-        <v>844</v>
-      </c>
-      <c r="H184" s="4" t="s">
-        <v>845</v>
-      </c>
-      <c r="I184" t="s">
-        <v>820</v>
-      </c>
-      <c r="K184" s="6" t="s">
-        <v>846</v>
-      </c>
-      <c r="L184" s="7" t="s">
-        <v>847</v>
-      </c>
-    </row>
-    <row r="185" spans="1:12">
-      <c r="A185" t="s">
-        <v>621</v>
-      </c>
-      <c r="B185" t="s">
-        <v>843</v>
-      </c>
-      <c r="D185" t="s">
-        <v>840</v>
-      </c>
-      <c r="E185" t="s">
-        <v>840</v>
-      </c>
-      <c r="F185" t="s">
-        <v>840</v>
-      </c>
-      <c r="G185" t="s">
-        <v>848</v>
-      </c>
-      <c r="H185" s="4" t="s">
-        <v>849</v>
-      </c>
-      <c r="I185" t="s">
-        <v>299</v>
-      </c>
-      <c r="K185" s="6" t="s">
-        <v>850</v>
-      </c>
-      <c r="L185" s="7" t="s">
-        <v>851</v>
       </c>
     </row>
     <row r="186" spans="1:12">
@@ -8983,19 +9046,19 @@
         <v>840</v>
       </c>
       <c r="G186" t="s">
-        <v>428</v>
+        <v>844</v>
       </c>
       <c r="H186" s="4" t="s">
-        <v>852</v>
+        <v>845</v>
       </c>
       <c r="I186" t="s">
-        <v>767</v>
+        <v>820</v>
       </c>
       <c r="K186" s="6" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
       <c r="L186" s="7" t="s">
-        <v>854</v>
+        <v>847</v>
       </c>
     </row>
     <row r="187" spans="1:12">
@@ -9015,19 +9078,19 @@
         <v>840</v>
       </c>
       <c r="G187" t="s">
-        <v>855</v>
+        <v>848</v>
       </c>
       <c r="H187" s="4" t="s">
-        <v>856</v>
+        <v>849</v>
       </c>
       <c r="I187" t="s">
-        <v>857</v>
+        <v>299</v>
       </c>
       <c r="K187" s="6" t="s">
-        <v>858</v>
+        <v>850</v>
       </c>
       <c r="L187" s="7" t="s">
-        <v>859</v>
+        <v>851</v>
       </c>
     </row>
     <row r="188" spans="1:12">
@@ -9035,7 +9098,7 @@
         <v>621</v>
       </c>
       <c r="B188" t="s">
-        <v>860</v>
+        <v>843</v>
       </c>
       <c r="D188" t="s">
         <v>840</v>
@@ -9047,19 +9110,19 @@
         <v>840</v>
       </c>
       <c r="G188" t="s">
-        <v>861</v>
+        <v>428</v>
       </c>
       <c r="H188" s="4" t="s">
-        <v>862</v>
+        <v>852</v>
       </c>
       <c r="I188" t="s">
-        <v>863</v>
+        <v>767</v>
       </c>
       <c r="K188" s="6" t="s">
-        <v>864</v>
+        <v>853</v>
       </c>
       <c r="L188" s="7" t="s">
-        <v>865</v>
+        <v>854</v>
       </c>
     </row>
     <row r="189" spans="1:12">
@@ -9067,7 +9130,7 @@
         <v>621</v>
       </c>
       <c r="B189" t="s">
-        <v>860</v>
+        <v>843</v>
       </c>
       <c r="D189" t="s">
         <v>840</v>
@@ -9079,19 +9142,19 @@
         <v>840</v>
       </c>
       <c r="G189" t="s">
-        <v>866</v>
+        <v>855</v>
       </c>
       <c r="H189" s="4" t="s">
-        <v>867</v>
+        <v>856</v>
       </c>
       <c r="I189" t="s">
-        <v>868</v>
-      </c>
-      <c r="K189" s="8" t="s">
-        <v>869</v>
+        <v>857</v>
+      </c>
+      <c r="K189" s="6" t="s">
+        <v>858</v>
       </c>
       <c r="L189" s="7" t="s">
-        <v>847</v>
+        <v>859</v>
       </c>
     </row>
     <row r="190" spans="1:12">
@@ -9099,7 +9162,7 @@
         <v>621</v>
       </c>
       <c r="B190" t="s">
-        <v>870</v>
+        <v>860</v>
       </c>
       <c r="D190" t="s">
         <v>840</v>
@@ -9111,22 +9174,19 @@
         <v>840</v>
       </c>
       <c r="G190" t="s">
-        <v>871</v>
+        <v>861</v>
       </c>
       <c r="H190" s="4" t="s">
-        <v>872</v>
+        <v>862</v>
       </c>
       <c r="I190" t="s">
-        <v>873</v>
-      </c>
-      <c r="J190" t="s">
-        <v>874</v>
+        <v>863</v>
       </c>
       <c r="K190" s="6" t="s">
-        <v>875</v>
+        <v>864</v>
       </c>
       <c r="L190" s="7" t="s">
-        <v>876</v>
+        <v>865</v>
       </c>
     </row>
     <row r="191" spans="1:12">
@@ -9134,7 +9194,7 @@
         <v>621</v>
       </c>
       <c r="B191" t="s">
-        <v>877</v>
+        <v>860</v>
       </c>
       <c r="D191" t="s">
         <v>840</v>
@@ -9146,22 +9206,19 @@
         <v>840</v>
       </c>
       <c r="G191" t="s">
-        <v>878</v>
+        <v>866</v>
       </c>
       <c r="H191" s="4" t="s">
-        <v>879</v>
+        <v>867</v>
       </c>
       <c r="I191" t="s">
-        <v>880</v>
-      </c>
-      <c r="J191" t="s">
-        <v>881</v>
-      </c>
-      <c r="K191" s="6" t="s">
-        <v>882</v>
+        <v>868</v>
+      </c>
+      <c r="K191" s="8" t="s">
+        <v>869</v>
       </c>
       <c r="L191" s="7" t="s">
-        <v>883</v>
+        <v>847</v>
       </c>
     </row>
     <row r="192" spans="1:12">
@@ -9169,7 +9226,7 @@
         <v>621</v>
       </c>
       <c r="B192" t="s">
-        <v>877</v>
+        <v>870</v>
       </c>
       <c r="D192" t="s">
         <v>840</v>
@@ -9181,19 +9238,22 @@
         <v>840</v>
       </c>
       <c r="G192" t="s">
-        <v>884</v>
+        <v>871</v>
       </c>
       <c r="H192" s="4" t="s">
-        <v>885</v>
+        <v>872</v>
       </c>
       <c r="I192" t="s">
-        <v>886</v>
+        <v>873</v>
+      </c>
+      <c r="J192" t="s">
+        <v>874</v>
       </c>
       <c r="K192" s="6" t="s">
-        <v>887</v>
+        <v>875</v>
       </c>
       <c r="L192" s="7" t="s">
-        <v>859</v>
+        <v>876</v>
       </c>
     </row>
     <row r="193" spans="1:12">
@@ -9201,31 +9261,34 @@
         <v>621</v>
       </c>
       <c r="B193" t="s">
-        <v>888</v>
+        <v>877</v>
       </c>
       <c r="D193" t="s">
-        <v>889</v>
+        <v>840</v>
       </c>
       <c r="E193" t="s">
-        <v>889</v>
+        <v>840</v>
       </c>
       <c r="F193" t="s">
-        <v>889</v>
+        <v>840</v>
       </c>
       <c r="G193" t="s">
-        <v>890</v>
+        <v>878</v>
       </c>
       <c r="H193" s="4" t="s">
-        <v>891</v>
+        <v>879</v>
       </c>
       <c r="I193" t="s">
-        <v>892</v>
+        <v>880</v>
+      </c>
+      <c r="J193" t="s">
+        <v>881</v>
       </c>
       <c r="K193" s="6" t="s">
-        <v>893</v>
+        <v>882</v>
       </c>
       <c r="L193" s="7" t="s">
-        <v>894</v>
+        <v>883</v>
       </c>
     </row>
     <row r="194" spans="1:12">
@@ -9233,31 +9296,31 @@
         <v>621</v>
       </c>
       <c r="B194" t="s">
-        <v>895</v>
+        <v>877</v>
       </c>
       <c r="D194" t="s">
-        <v>889</v>
+        <v>840</v>
       </c>
       <c r="E194" t="s">
-        <v>889</v>
+        <v>840</v>
       </c>
       <c r="F194" t="s">
-        <v>896</v>
+        <v>840</v>
       </c>
       <c r="G194" t="s">
-        <v>897</v>
+        <v>884</v>
       </c>
       <c r="H194" s="4" t="s">
-        <v>898</v>
+        <v>885</v>
       </c>
       <c r="I194" t="s">
-        <v>233</v>
+        <v>886</v>
       </c>
       <c r="K194" s="6" t="s">
-        <v>899</v>
+        <v>887</v>
       </c>
       <c r="L194" s="7" t="s">
-        <v>900</v>
+        <v>859</v>
       </c>
     </row>
     <row r="195" spans="1:12">
@@ -9265,7 +9328,7 @@
         <v>621</v>
       </c>
       <c r="B195" t="s">
-        <v>901</v>
+        <v>888</v>
       </c>
       <c r="D195" t="s">
         <v>889</v>
@@ -9274,22 +9337,22 @@
         <v>889</v>
       </c>
       <c r="F195" t="s">
-        <v>896</v>
+        <v>889</v>
       </c>
       <c r="G195" t="s">
-        <v>902</v>
+        <v>890</v>
       </c>
       <c r="H195" s="4" t="s">
-        <v>903</v>
+        <v>891</v>
       </c>
       <c r="I195" t="s">
-        <v>904</v>
+        <v>892</v>
       </c>
       <c r="K195" s="6" t="s">
-        <v>905</v>
+        <v>893</v>
       </c>
       <c r="L195" s="7" t="s">
-        <v>791</v>
+        <v>894</v>
       </c>
     </row>
     <row r="196" spans="1:12">
@@ -9297,7 +9360,7 @@
         <v>621</v>
       </c>
       <c r="B196" t="s">
-        <v>906</v>
+        <v>895</v>
       </c>
       <c r="D196" t="s">
         <v>889</v>
@@ -9306,22 +9369,22 @@
         <v>889</v>
       </c>
       <c r="F196" t="s">
-        <v>907</v>
+        <v>896</v>
       </c>
       <c r="G196" t="s">
-        <v>908</v>
+        <v>897</v>
       </c>
       <c r="H196" s="4" t="s">
-        <v>909</v>
+        <v>898</v>
       </c>
       <c r="I196" t="s">
-        <v>910</v>
+        <v>233</v>
       </c>
       <c r="K196" s="6" t="s">
-        <v>911</v>
+        <v>899</v>
       </c>
       <c r="L196" s="7" t="s">
-        <v>912</v>
+        <v>900</v>
       </c>
     </row>
     <row r="197" spans="1:12">
@@ -9329,7 +9392,7 @@
         <v>621</v>
       </c>
       <c r="B197" t="s">
-        <v>906</v>
+        <v>901</v>
       </c>
       <c r="D197" t="s">
         <v>889</v>
@@ -9338,22 +9401,22 @@
         <v>889</v>
       </c>
       <c r="F197" t="s">
-        <v>907</v>
+        <v>896</v>
       </c>
       <c r="G197" t="s">
-        <v>913</v>
+        <v>902</v>
       </c>
       <c r="H197" s="4" t="s">
-        <v>914</v>
+        <v>903</v>
       </c>
       <c r="I197" t="s">
-        <v>915</v>
+        <v>904</v>
       </c>
       <c r="K197" s="6" t="s">
-        <v>916</v>
+        <v>905</v>
       </c>
       <c r="L197" s="7" t="s">
-        <v>917</v>
+        <v>791</v>
       </c>
     </row>
     <row r="198" spans="1:12">
@@ -9361,7 +9424,7 @@
         <v>621</v>
       </c>
       <c r="B198" t="s">
-        <v>918</v>
+        <v>906</v>
       </c>
       <c r="D198" t="s">
         <v>889</v>
@@ -9373,19 +9436,19 @@
         <v>907</v>
       </c>
       <c r="G198" t="s">
-        <v>919</v>
+        <v>908</v>
       </c>
       <c r="H198" s="4" t="s">
-        <v>920</v>
+        <v>909</v>
       </c>
       <c r="I198" t="s">
-        <v>921</v>
+        <v>910</v>
       </c>
       <c r="K198" s="6" t="s">
-        <v>922</v>
+        <v>911</v>
       </c>
       <c r="L198" s="7" t="s">
-        <v>917</v>
+        <v>912</v>
       </c>
     </row>
     <row r="199" spans="1:12">
@@ -9393,7 +9456,7 @@
         <v>621</v>
       </c>
       <c r="B199" t="s">
-        <v>923</v>
+        <v>906</v>
       </c>
       <c r="D199" t="s">
         <v>889</v>
@@ -9402,22 +9465,22 @@
         <v>889</v>
       </c>
       <c r="F199" t="s">
-        <v>924</v>
+        <v>907</v>
       </c>
       <c r="G199" t="s">
-        <v>925</v>
+        <v>913</v>
       </c>
       <c r="H199" s="4" t="s">
-        <v>926</v>
+        <v>914</v>
       </c>
       <c r="I199" t="s">
-        <v>927</v>
+        <v>915</v>
       </c>
       <c r="K199" s="6" t="s">
-        <v>928</v>
+        <v>916</v>
       </c>
       <c r="L199" s="7" t="s">
-        <v>929</v>
+        <v>917</v>
       </c>
     </row>
     <row r="200" spans="1:12">
@@ -9425,31 +9488,31 @@
         <v>621</v>
       </c>
       <c r="B200" t="s">
-        <v>930</v>
+        <v>918</v>
       </c>
       <c r="D200" t="s">
-        <v>931</v>
+        <v>889</v>
       </c>
       <c r="E200" t="s">
-        <v>931</v>
+        <v>889</v>
       </c>
       <c r="F200" t="s">
-        <v>932</v>
+        <v>907</v>
       </c>
       <c r="G200" t="s">
-        <v>933</v>
+        <v>919</v>
       </c>
       <c r="H200" s="4" t="s">
-        <v>934</v>
+        <v>920</v>
       </c>
       <c r="I200" t="s">
-        <v>935</v>
+        <v>921</v>
       </c>
       <c r="K200" s="6" t="s">
-        <v>936</v>
+        <v>922</v>
       </c>
       <c r="L200" s="7" t="s">
-        <v>937</v>
+        <v>917</v>
       </c>
     </row>
     <row r="201" spans="1:12">
@@ -9457,34 +9520,31 @@
         <v>621</v>
       </c>
       <c r="B201" t="s">
-        <v>938</v>
+        <v>923</v>
       </c>
       <c r="D201" t="s">
-        <v>931</v>
+        <v>889</v>
       </c>
       <c r="E201" t="s">
-        <v>931</v>
+        <v>889</v>
       </c>
       <c r="F201" t="s">
-        <v>939</v>
+        <v>924</v>
       </c>
       <c r="G201" t="s">
-        <v>940</v>
+        <v>925</v>
       </c>
       <c r="H201" s="4" t="s">
-        <v>941</v>
+        <v>926</v>
       </c>
       <c r="I201" t="s">
-        <v>99</v>
-      </c>
-      <c r="J201" t="s">
-        <v>942</v>
-      </c>
-      <c r="K201" s="8" t="s">
-        <v>943</v>
+        <v>927</v>
+      </c>
+      <c r="K201" s="6" t="s">
+        <v>928</v>
       </c>
       <c r="L201" s="7" t="s">
-        <v>944</v>
+        <v>929</v>
       </c>
     </row>
     <row r="202" spans="1:12">
@@ -9492,7 +9552,7 @@
         <v>621</v>
       </c>
       <c r="B202" t="s">
-        <v>945</v>
+        <v>930</v>
       </c>
       <c r="D202" t="s">
         <v>931</v>
@@ -9501,22 +9561,22 @@
         <v>931</v>
       </c>
       <c r="F202" t="s">
-        <v>939</v>
+        <v>932</v>
       </c>
       <c r="G202" t="s">
-        <v>946</v>
+        <v>933</v>
       </c>
       <c r="H202" s="4" t="s">
-        <v>947</v>
+        <v>934</v>
       </c>
       <c r="I202" t="s">
-        <v>314</v>
+        <v>935</v>
       </c>
       <c r="K202" s="6" t="s">
-        <v>948</v>
+        <v>936</v>
       </c>
       <c r="L202" s="7" t="s">
-        <v>949</v>
+        <v>937</v>
       </c>
     </row>
     <row r="203" spans="1:12">
@@ -9524,7 +9584,7 @@
         <v>621</v>
       </c>
       <c r="B203" t="s">
-        <v>945</v>
+        <v>938</v>
       </c>
       <c r="D203" t="s">
         <v>931</v>
@@ -9536,19 +9596,22 @@
         <v>939</v>
       </c>
       <c r="G203" t="s">
-        <v>950</v>
+        <v>940</v>
       </c>
       <c r="H203" s="4" t="s">
-        <v>951</v>
+        <v>941</v>
       </c>
       <c r="I203" t="s">
-        <v>221</v>
-      </c>
-      <c r="K203" s="6" t="s">
-        <v>952</v>
+        <v>99</v>
+      </c>
+      <c r="J203" t="s">
+        <v>942</v>
+      </c>
+      <c r="K203" s="8" t="s">
+        <v>943</v>
       </c>
       <c r="L203" s="7" t="s">
-        <v>953</v>
+        <v>944</v>
       </c>
     </row>
     <row r="204" spans="1:12">
@@ -9556,7 +9619,7 @@
         <v>621</v>
       </c>
       <c r="B204" t="s">
-        <v>954</v>
+        <v>945</v>
       </c>
       <c r="D204" t="s">
         <v>931</v>
@@ -9565,22 +9628,22 @@
         <v>931</v>
       </c>
       <c r="F204" t="s">
-        <v>932</v>
+        <v>939</v>
       </c>
       <c r="G204" t="s">
-        <v>955</v>
+        <v>946</v>
       </c>
       <c r="H204" s="4" t="s">
-        <v>956</v>
+        <v>947</v>
       </c>
       <c r="I204" t="s">
-        <v>767</v>
+        <v>314</v>
       </c>
       <c r="K204" s="6" t="s">
-        <v>957</v>
+        <v>948</v>
       </c>
       <c r="L204" s="7" t="s">
-        <v>958</v>
+        <v>949</v>
       </c>
     </row>
     <row r="205" spans="1:12">
@@ -9588,7 +9651,7 @@
         <v>621</v>
       </c>
       <c r="B205" t="s">
-        <v>959</v>
+        <v>945</v>
       </c>
       <c r="D205" t="s">
         <v>931</v>
@@ -9600,19 +9663,19 @@
         <v>939</v>
       </c>
       <c r="G205" t="s">
-        <v>960</v>
+        <v>950</v>
       </c>
       <c r="H205" s="4" t="s">
-        <v>961</v>
+        <v>951</v>
       </c>
       <c r="I205" t="s">
-        <v>962</v>
+        <v>221</v>
       </c>
       <c r="K205" s="6" t="s">
-        <v>963</v>
+        <v>952</v>
       </c>
       <c r="L205" s="7" t="s">
-        <v>964</v>
+        <v>953</v>
       </c>
     </row>
     <row r="206" spans="1:12">
@@ -9620,7 +9683,7 @@
         <v>621</v>
       </c>
       <c r="B206" t="s">
-        <v>959</v>
+        <v>954</v>
       </c>
       <c r="D206" t="s">
         <v>931</v>
@@ -9629,22 +9692,22 @@
         <v>931</v>
       </c>
       <c r="F206" t="s">
-        <v>939</v>
+        <v>932</v>
       </c>
       <c r="G206" t="s">
-        <v>965</v>
+        <v>955</v>
       </c>
       <c r="H206" s="4" t="s">
-        <v>966</v>
+        <v>956</v>
       </c>
       <c r="I206" t="s">
-        <v>801</v>
+        <v>767</v>
       </c>
       <c r="K206" s="6" t="s">
-        <v>967</v>
+        <v>957</v>
       </c>
       <c r="L206" s="7" t="s">
-        <v>953</v>
+        <v>958</v>
       </c>
     </row>
     <row r="207" spans="1:12">
@@ -9652,7 +9715,7 @@
         <v>621</v>
       </c>
       <c r="B207" t="s">
-        <v>189</v>
+        <v>959</v>
       </c>
       <c r="D207" t="s">
         <v>931</v>
@@ -9661,25 +9724,22 @@
         <v>931</v>
       </c>
       <c r="F207" t="s">
-        <v>932</v>
+        <v>939</v>
       </c>
       <c r="G207" t="s">
-        <v>968</v>
+        <v>960</v>
       </c>
       <c r="H207" s="4" t="s">
-        <v>969</v>
+        <v>961</v>
       </c>
       <c r="I207" t="s">
-        <v>970</v>
-      </c>
-      <c r="J207" t="s">
-        <v>971</v>
+        <v>962</v>
       </c>
       <c r="K207" s="6" t="s">
-        <v>972</v>
+        <v>963</v>
       </c>
       <c r="L207" s="7" t="s">
-        <v>973</v>
+        <v>964</v>
       </c>
     </row>
     <row r="208" spans="1:12">
@@ -9687,7 +9747,7 @@
         <v>621</v>
       </c>
       <c r="B208" t="s">
-        <v>974</v>
+        <v>959</v>
       </c>
       <c r="D208" t="s">
         <v>931</v>
@@ -9696,22 +9756,22 @@
         <v>931</v>
       </c>
       <c r="F208" t="s">
-        <v>932</v>
+        <v>939</v>
       </c>
       <c r="G208" t="s">
-        <v>975</v>
+        <v>965</v>
       </c>
       <c r="H208" s="4" t="s">
-        <v>976</v>
+        <v>966</v>
       </c>
       <c r="I208" t="s">
-        <v>977</v>
+        <v>801</v>
       </c>
       <c r="K208" s="6" t="s">
-        <v>978</v>
+        <v>967</v>
       </c>
       <c r="L208" s="7" t="s">
-        <v>979</v>
+        <v>953</v>
       </c>
     </row>
     <row r="209" spans="1:13">
@@ -9719,7 +9779,7 @@
         <v>621</v>
       </c>
       <c r="B209" t="s">
-        <v>974</v>
+        <v>189</v>
       </c>
       <c r="D209" t="s">
         <v>931</v>
@@ -9731,19 +9791,22 @@
         <v>932</v>
       </c>
       <c r="G209" t="s">
-        <v>980</v>
+        <v>968</v>
       </c>
       <c r="H209" s="4" t="s">
-        <v>981</v>
+        <v>969</v>
       </c>
       <c r="I209" t="s">
-        <v>982</v>
+        <v>970</v>
+      </c>
+      <c r="J209" t="s">
+        <v>971</v>
       </c>
       <c r="K209" s="6" t="s">
-        <v>983</v>
+        <v>972</v>
       </c>
       <c r="L209" s="7" t="s">
-        <v>984</v>
+        <v>973</v>
       </c>
     </row>
     <row r="210" spans="1:13">
@@ -9751,31 +9814,31 @@
         <v>621</v>
       </c>
       <c r="B210" t="s">
-        <v>51</v>
+        <v>974</v>
       </c>
       <c r="D210" t="s">
-        <v>985</v>
+        <v>931</v>
       </c>
       <c r="E210" t="s">
-        <v>985</v>
+        <v>931</v>
       </c>
       <c r="F210" t="s">
-        <v>986</v>
+        <v>932</v>
       </c>
       <c r="G210" t="s">
-        <v>987</v>
+        <v>975</v>
       </c>
       <c r="H210" s="4" t="s">
-        <v>988</v>
+        <v>976</v>
       </c>
       <c r="I210" t="s">
-        <v>989</v>
-      </c>
-      <c r="K210" s="8" t="s">
-        <v>990</v>
+        <v>977</v>
+      </c>
+      <c r="K210" s="6" t="s">
+        <v>978</v>
       </c>
       <c r="L210" s="7" t="s">
-        <v>991</v>
+        <v>979</v>
       </c>
     </row>
     <row r="211" spans="1:13">
@@ -9783,39 +9846,39 @@
         <v>621</v>
       </c>
       <c r="B211" t="s">
-        <v>992</v>
+        <v>974</v>
       </c>
       <c r="D211" t="s">
-        <v>985</v>
+        <v>931</v>
       </c>
       <c r="E211" t="s">
-        <v>985</v>
+        <v>931</v>
       </c>
       <c r="F211" t="s">
-        <v>986</v>
+        <v>932</v>
       </c>
       <c r="G211" t="s">
-        <v>987</v>
+        <v>980</v>
       </c>
       <c r="H211" s="4" t="s">
-        <v>988</v>
+        <v>981</v>
       </c>
       <c r="I211" t="s">
-        <v>989</v>
-      </c>
-      <c r="K211" s="8" t="s">
-        <v>990</v>
+        <v>982</v>
+      </c>
+      <c r="K211" s="6" t="s">
+        <v>983</v>
       </c>
       <c r="L211" s="7" t="s">
-        <v>991</v>
+        <v>984</v>
       </c>
     </row>
     <row r="212" spans="1:13">
       <c r="A212" t="s">
         <v>621</v>
       </c>
-      <c r="B212">
-        <v>147</v>
+      <c r="B212" t="s">
+        <v>51</v>
       </c>
       <c r="D212" t="s">
         <v>985</v>
@@ -9824,25 +9887,22 @@
         <v>985</v>
       </c>
       <c r="F212" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="G212" t="s">
-        <v>993</v>
+        <v>987</v>
       </c>
       <c r="H212" s="4" t="s">
-        <v>994</v>
+        <v>988</v>
       </c>
       <c r="I212" t="s">
-        <v>767</v>
-      </c>
-      <c r="J212" t="s">
-        <v>995</v>
-      </c>
-      <c r="K212" s="6" t="s">
-        <v>996</v>
+        <v>989</v>
+      </c>
+      <c r="K212" s="8" t="s">
+        <v>990</v>
       </c>
       <c r="L212" s="7" t="s">
-        <v>997</v>
+        <v>991</v>
       </c>
     </row>
     <row r="213" spans="1:13">
@@ -9850,107 +9910,106 @@
         <v>621</v>
       </c>
       <c r="B213" t="s">
+        <v>992</v>
+      </c>
+      <c r="D213" t="s">
+        <v>985</v>
+      </c>
+      <c r="E213" t="s">
+        <v>985</v>
+      </c>
+      <c r="F213" t="s">
+        <v>986</v>
+      </c>
+      <c r="G213" t="s">
+        <v>987</v>
+      </c>
+      <c r="H213" s="4" t="s">
+        <v>988</v>
+      </c>
+      <c r="I213" t="s">
+        <v>989</v>
+      </c>
+      <c r="K213" s="8" t="s">
+        <v>990</v>
+      </c>
+      <c r="L213" s="7" t="s">
+        <v>991</v>
+      </c>
+    </row>
+    <row r="214" spans="1:13">
+      <c r="A214" t="s">
+        <v>621</v>
+      </c>
+      <c r="B214">
+        <v>147</v>
+      </c>
+      <c r="D214" t="s">
+        <v>985</v>
+      </c>
+      <c r="E214" t="s">
+        <v>985</v>
+      </c>
+      <c r="F214" t="s">
+        <v>985</v>
+      </c>
+      <c r="G214" t="s">
+        <v>993</v>
+      </c>
+      <c r="H214" s="4" t="s">
+        <v>994</v>
+      </c>
+      <c r="I214" t="s">
+        <v>767</v>
+      </c>
+      <c r="J214" t="s">
+        <v>995</v>
+      </c>
+      <c r="K214" s="6" t="s">
+        <v>996</v>
+      </c>
+      <c r="L214" s="7" t="s">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="215" spans="1:13">
+      <c r="A215" t="s">
+        <v>621</v>
+      </c>
+      <c r="B215" t="s">
         <v>998</v>
       </c>
-      <c r="D213" t="s">
+      <c r="D215" t="s">
         <v>999</v>
       </c>
-      <c r="E213" t="s">
+      <c r="E215" t="s">
         <v>999</v>
       </c>
-      <c r="F213" t="s">
+      <c r="F215" t="s">
         <v>999</v>
       </c>
-      <c r="G213" s="27" t="s">
+      <c r="G215" s="27" t="s">
         <v>658</v>
       </c>
-      <c r="H213" s="4" t="s">
+      <c r="H215" s="4" t="s">
         <v>659</v>
       </c>
-      <c r="I213" t="s">
+      <c r="I215" t="s">
         <v>338</v>
       </c>
-      <c r="K213" s="6" t="s">
+      <c r="K215" s="6" t="s">
         <v>660</v>
       </c>
-      <c r="L213" s="7" t="s">
+      <c r="L215" s="7" t="s">
         <v>661</v>
       </c>
     </row>
-    <row r="214" spans="1:13" ht="15.6">
-      <c r="A214" t="s">
-        <v>621</v>
-      </c>
-      <c r="B214" t="s">
+    <row r="216" spans="1:13" ht="15.5">
+      <c r="A216" t="s">
+        <v>621</v>
+      </c>
+      <c r="B216" t="s">
         <v>998</v>
-      </c>
-      <c r="D214" t="s">
-        <v>999</v>
-      </c>
-      <c r="E214" t="s">
-        <v>999</v>
-      </c>
-      <c r="F214" t="s">
-        <v>999</v>
-      </c>
-      <c r="G214" t="s">
-        <v>1000</v>
-      </c>
-      <c r="H214" s="4" t="s">
-        <v>1001</v>
-      </c>
-      <c r="I214" t="s">
-        <v>1002</v>
-      </c>
-      <c r="K214" s="8" t="s">
-        <v>1003</v>
-      </c>
-      <c r="L214" s="12" t="s">
-        <v>1004</v>
-      </c>
-    </row>
-    <row r="215" spans="1:13" ht="15.6">
-      <c r="A215" s="23" t="s">
-        <v>621</v>
-      </c>
-      <c r="B215" s="23" t="s">
-        <v>998</v>
-      </c>
-      <c r="C215" s="23"/>
-      <c r="D215" s="23" t="s">
-        <v>999</v>
-      </c>
-      <c r="E215" s="23" t="s">
-        <v>999</v>
-      </c>
-      <c r="F215" s="23" t="s">
-        <v>999</v>
-      </c>
-      <c r="G215" s="23" t="s">
-        <v>913</v>
-      </c>
-      <c r="H215" s="24" t="s">
-        <v>761</v>
-      </c>
-      <c r="I215" s="23" t="s">
-        <v>1127</v>
-      </c>
-      <c r="J215" s="23" t="s">
-        <v>1128</v>
-      </c>
-      <c r="K215" s="25" t="s">
-        <v>1130</v>
-      </c>
-      <c r="L215" s="26" t="s">
-        <v>1129</v>
-      </c>
-    </row>
-    <row r="216" spans="1:13">
-      <c r="A216" t="s">
-        <v>621</v>
-      </c>
-      <c r="B216" t="s">
-        <v>1005</v>
       </c>
       <c r="D216" t="s">
         <v>999</v>
@@ -9962,54 +10021,55 @@
         <v>999</v>
       </c>
       <c r="G216" t="s">
-        <v>1006</v>
+        <v>1000</v>
       </c>
       <c r="H216" s="4" t="s">
-        <v>1007</v>
+        <v>1001</v>
       </c>
       <c r="I216" t="s">
-        <v>1008</v>
-      </c>
-      <c r="J216" t="s">
-        <v>1009</v>
-      </c>
-      <c r="K216" s="6" t="s">
-        <v>1010</v>
-      </c>
-      <c r="L216" s="7" t="s">
-        <v>1011</v>
-      </c>
-    </row>
-    <row r="217" spans="1:13">
-      <c r="A217" t="s">
-        <v>621</v>
-      </c>
-      <c r="B217">
-        <v>145</v>
-      </c>
-      <c r="D217" t="s">
-        <v>1012</v>
-      </c>
-      <c r="E217" t="s">
-        <v>1012</v>
-      </c>
-      <c r="F217" t="s">
-        <v>1012</v>
-      </c>
-      <c r="G217" t="s">
-        <v>1013</v>
-      </c>
-      <c r="H217" s="4" t="s">
-        <v>1014</v>
-      </c>
-      <c r="I217" t="s">
-        <v>1015</v>
-      </c>
-      <c r="K217" s="6" t="s">
-        <v>1016</v>
-      </c>
-      <c r="L217" s="9" t="s">
-        <v>490</v>
+        <v>1002</v>
+      </c>
+      <c r="K216" s="8" t="s">
+        <v>1003</v>
+      </c>
+      <c r="L216" s="12" t="s">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="217" spans="1:13" ht="15.5">
+      <c r="A217" s="23" t="s">
+        <v>621</v>
+      </c>
+      <c r="B217" s="23" t="s">
+        <v>998</v>
+      </c>
+      <c r="C217" s="23"/>
+      <c r="D217" s="23" t="s">
+        <v>999</v>
+      </c>
+      <c r="E217" s="23" t="s">
+        <v>999</v>
+      </c>
+      <c r="F217" s="23" t="s">
+        <v>999</v>
+      </c>
+      <c r="G217" s="23" t="s">
+        <v>913</v>
+      </c>
+      <c r="H217" s="24" t="s">
+        <v>761</v>
+      </c>
+      <c r="I217" s="23" t="s">
+        <v>1127</v>
+      </c>
+      <c r="J217" s="23" t="s">
+        <v>1128</v>
+      </c>
+      <c r="K217" s="25" t="s">
+        <v>1130</v>
+      </c>
+      <c r="L217" s="26" t="s">
+        <v>1129</v>
       </c>
     </row>
     <row r="218" spans="1:13">
@@ -10017,66 +10077,66 @@
         <v>621</v>
       </c>
       <c r="B218" t="s">
-        <v>1017</v>
+        <v>1005</v>
       </c>
       <c r="D218" t="s">
-        <v>1018</v>
+        <v>999</v>
       </c>
       <c r="E218" t="s">
-        <v>1018</v>
+        <v>999</v>
       </c>
       <c r="F218" t="s">
-        <v>1018</v>
+        <v>999</v>
       </c>
       <c r="G218" t="s">
-        <v>1019</v>
+        <v>1006</v>
       </c>
       <c r="H218" s="4" t="s">
-        <v>761</v>
+        <v>1007</v>
       </c>
       <c r="I218" t="s">
-        <v>1020</v>
+        <v>1008</v>
       </c>
       <c r="J218" t="s">
-        <v>1021</v>
+        <v>1009</v>
+      </c>
+      <c r="K218" s="6" t="s">
+        <v>1010</v>
       </c>
       <c r="L218" s="7" t="s">
-        <v>764</v>
-      </c>
-      <c r="M218" t="s">
-        <v>1022</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="219" spans="1:13">
       <c r="A219" t="s">
         <v>621</v>
       </c>
-      <c r="B219" t="s">
-        <v>1017</v>
+      <c r="B219">
+        <v>145</v>
       </c>
       <c r="D219" t="s">
-        <v>1018</v>
+        <v>1012</v>
       </c>
       <c r="E219" t="s">
-        <v>1018</v>
+        <v>1012</v>
       </c>
       <c r="F219" t="s">
-        <v>1018</v>
+        <v>1012</v>
       </c>
       <c r="G219" t="s">
-        <v>1023</v>
+        <v>1013</v>
       </c>
       <c r="H219" s="4" t="s">
-        <v>761</v>
+        <v>1014</v>
       </c>
       <c r="I219" t="s">
-        <v>383</v>
-      </c>
-      <c r="K219" t="s">
-        <v>1117</v>
-      </c>
-      <c r="L219" s="7" t="s">
-        <v>1119</v>
+        <v>1015</v>
+      </c>
+      <c r="K219" s="6" t="s">
+        <v>1016</v>
+      </c>
+      <c r="L219" s="9" t="s">
+        <v>490</v>
       </c>
     </row>
     <row r="220" spans="1:13">
@@ -10084,7 +10144,7 @@
         <v>621</v>
       </c>
       <c r="B220" t="s">
-        <v>1024</v>
+        <v>1017</v>
       </c>
       <c r="D220" t="s">
         <v>1018</v>
@@ -10096,30 +10156,30 @@
         <v>1018</v>
       </c>
       <c r="G220" t="s">
-        <v>1025</v>
+        <v>1019</v>
       </c>
       <c r="H220" s="4" t="s">
         <v>761</v>
       </c>
       <c r="I220" t="s">
-        <v>1026</v>
+        <v>1020</v>
       </c>
       <c r="J220" t="s">
-        <v>1027</v>
-      </c>
-      <c r="K220" t="s">
-        <v>1116</v>
+        <v>1021</v>
       </c>
       <c r="L220" s="7" t="s">
         <v>764</v>
       </c>
+      <c r="M220" t="s">
+        <v>1022</v>
+      </c>
     </row>
     <row r="221" spans="1:13">
       <c r="A221" t="s">
         <v>621</v>
       </c>
       <c r="B221" t="s">
-        <v>1028</v>
+        <v>1017</v>
       </c>
       <c r="D221" t="s">
         <v>1018</v>
@@ -10131,19 +10191,19 @@
         <v>1018</v>
       </c>
       <c r="G221" t="s">
-        <v>1029</v>
+        <v>1023</v>
       </c>
       <c r="H221" s="4" t="s">
-        <v>1120</v>
+        <v>761</v>
       </c>
       <c r="I221" t="s">
-        <v>1030</v>
+        <v>383</v>
       </c>
       <c r="K221" t="s">
-        <v>1121</v>
+        <v>1117</v>
       </c>
       <c r="L221" s="7" t="s">
-        <v>375</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="222" spans="1:13">
@@ -10151,7 +10211,7 @@
         <v>621</v>
       </c>
       <c r="B222" t="s">
-        <v>1031</v>
+        <v>1024</v>
       </c>
       <c r="D222" t="s">
         <v>1018</v>
@@ -10163,20 +10223,30 @@
         <v>1018</v>
       </c>
       <c r="G222" t="s">
-        <v>1032</v>
-      </c>
-      <c r="H222" s="4"/>
+        <v>1025</v>
+      </c>
+      <c r="H222" s="4" t="s">
+        <v>761</v>
+      </c>
       <c r="I222" t="s">
-        <v>1018</v>
-      </c>
-      <c r="L222" s="7"/>
+        <v>1026</v>
+      </c>
+      <c r="J222" t="s">
+        <v>1027</v>
+      </c>
+      <c r="K222" t="s">
+        <v>1116</v>
+      </c>
+      <c r="L222" s="7" t="s">
+        <v>764</v>
+      </c>
     </row>
     <row r="223" spans="1:13">
       <c r="A223" t="s">
         <v>621</v>
       </c>
       <c r="B223" t="s">
-        <v>1033</v>
+        <v>1028</v>
       </c>
       <c r="D223" t="s">
         <v>1018</v>
@@ -10188,19 +10258,19 @@
         <v>1018</v>
       </c>
       <c r="G223" t="s">
-        <v>1034</v>
+        <v>1029</v>
       </c>
       <c r="H223" s="4" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
       <c r="I223" t="s">
-        <v>1035</v>
+        <v>1030</v>
       </c>
       <c r="K223" t="s">
-        <v>1118</v>
+        <v>1121</v>
       </c>
       <c r="L223" s="7" t="s">
-        <v>1123</v>
+        <v>375</v>
       </c>
     </row>
     <row r="224" spans="1:13">
@@ -10208,7 +10278,7 @@
         <v>621</v>
       </c>
       <c r="B224" t="s">
-        <v>1036</v>
+        <v>1031</v>
       </c>
       <c r="D224" t="s">
         <v>1018</v>
@@ -10219,13 +10289,13 @@
       <c r="F224" t="s">
         <v>1018</v>
       </c>
-      <c r="G224" s="22" t="s">
-        <v>1109</v>
-      </c>
-      <c r="H224" s="5"/>
-      <c r="I224" s="19"/>
-      <c r="J224" s="19"/>
-      <c r="K224" s="20"/>
+      <c r="G224" t="s">
+        <v>1032</v>
+      </c>
+      <c r="H224" s="4"/>
+      <c r="I224" t="s">
+        <v>1018</v>
+      </c>
       <c r="L224" s="7"/>
     </row>
     <row r="225" spans="1:12">
@@ -10233,7 +10303,7 @@
         <v>621</v>
       </c>
       <c r="B225" t="s">
-        <v>1037</v>
+        <v>1033</v>
       </c>
       <c r="D225" t="s">
         <v>1018</v>
@@ -10245,19 +10315,19 @@
         <v>1018</v>
       </c>
       <c r="G225" t="s">
-        <v>1038</v>
+        <v>1034</v>
       </c>
       <c r="H225" s="4" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
       <c r="I225" t="s">
-        <v>1039</v>
-      </c>
-      <c r="K225" s="18" t="s">
-        <v>1109</v>
+        <v>1035</v>
+      </c>
+      <c r="K225" t="s">
+        <v>1118</v>
       </c>
       <c r="L225" s="7" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="226" spans="1:12">
@@ -10265,24 +10335,24 @@
         <v>621</v>
       </c>
       <c r="B226" t="s">
-        <v>1040</v>
+        <v>1036</v>
       </c>
       <c r="D226" t="s">
-        <v>985</v>
+        <v>1018</v>
       </c>
       <c r="E226" t="s">
-        <v>985</v>
+        <v>1018</v>
       </c>
       <c r="F226" t="s">
-        <v>985</v>
-      </c>
-      <c r="G226" t="s">
-        <v>1041</v>
-      </c>
-      <c r="H226" s="4"/>
-      <c r="I226" t="s">
-        <v>1042</v>
-      </c>
+        <v>1018</v>
+      </c>
+      <c r="G226" s="22" t="s">
+        <v>1109</v>
+      </c>
+      <c r="H226" s="5"/>
+      <c r="I226" s="19"/>
+      <c r="J226" s="19"/>
+      <c r="K226" s="20"/>
       <c r="L226" s="7"/>
     </row>
     <row r="227" spans="1:12">
@@ -10290,32 +10360,39 @@
         <v>621</v>
       </c>
       <c r="B227" t="s">
-        <v>1043</v>
+        <v>1037</v>
       </c>
       <c r="D227" t="s">
-        <v>985</v>
+        <v>1018</v>
       </c>
       <c r="E227" t="s">
-        <v>985</v>
+        <v>1018</v>
       </c>
       <c r="F227" t="s">
-        <v>985</v>
+        <v>1018</v>
       </c>
       <c r="G227" t="s">
-        <v>1044</v>
-      </c>
-      <c r="H227" s="4"/>
+        <v>1038</v>
+      </c>
+      <c r="H227" s="4" t="s">
+        <v>1124</v>
+      </c>
       <c r="I227" t="s">
-        <v>1045</v>
-      </c>
-      <c r="L227" s="7"/>
+        <v>1039</v>
+      </c>
+      <c r="K227" s="18" t="s">
+        <v>1109</v>
+      </c>
+      <c r="L227" s="7" t="s">
+        <v>1125</v>
+      </c>
     </row>
     <row r="228" spans="1:12">
       <c r="A228" t="s">
         <v>621</v>
       </c>
       <c r="B228" t="s">
-        <v>1046</v>
+        <v>1040</v>
       </c>
       <c r="D228" t="s">
         <v>985</v>
@@ -10327,7 +10404,7 @@
         <v>985</v>
       </c>
       <c r="G228" t="s">
-        <v>1047</v>
+        <v>1041</v>
       </c>
       <c r="H228" s="4"/>
       <c r="I228" t="s">
@@ -10340,7 +10417,7 @@
         <v>621</v>
       </c>
       <c r="B229" t="s">
-        <v>1048</v>
+        <v>1043</v>
       </c>
       <c r="D229" t="s">
         <v>985</v>
@@ -10352,11 +10429,11 @@
         <v>985</v>
       </c>
       <c r="G229" t="s">
-        <v>1049</v>
+        <v>1044</v>
       </c>
       <c r="H229" s="4"/>
       <c r="I229" t="s">
-        <v>1042</v>
+        <v>1045</v>
       </c>
       <c r="L229" s="7"/>
     </row>
@@ -10365,7 +10442,7 @@
         <v>621</v>
       </c>
       <c r="B230" t="s">
-        <v>1050</v>
+        <v>1046</v>
       </c>
       <c r="D230" t="s">
         <v>985</v>
@@ -10377,7 +10454,7 @@
         <v>985</v>
       </c>
       <c r="G230" t="s">
-        <v>1051</v>
+        <v>1047</v>
       </c>
       <c r="H230" s="4"/>
       <c r="I230" t="s">
@@ -10390,49 +10467,44 @@
         <v>621</v>
       </c>
       <c r="B231" t="s">
-        <v>1052</v>
+        <v>1048</v>
       </c>
       <c r="D231" t="s">
-        <v>889</v>
+        <v>985</v>
       </c>
       <c r="E231" t="s">
-        <v>889</v>
+        <v>985</v>
       </c>
       <c r="F231" t="s">
-        <v>889</v>
+        <v>985</v>
       </c>
       <c r="G231" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
       <c r="H231" s="4"/>
       <c r="I231" t="s">
-        <v>233</v>
-      </c>
-      <c r="K231" s="6" t="s">
-        <v>899</v>
-      </c>
-      <c r="L231" s="7" t="s">
-        <v>900</v>
-      </c>
+        <v>1042</v>
+      </c>
+      <c r="L231" s="7"/>
     </row>
     <row r="232" spans="1:12">
       <c r="A232" t="s">
         <v>621</v>
       </c>
       <c r="B232" t="s">
-        <v>1054</v>
+        <v>1050</v>
       </c>
       <c r="D232" t="s">
-        <v>889</v>
+        <v>985</v>
       </c>
       <c r="E232" t="s">
-        <v>889</v>
+        <v>985</v>
       </c>
       <c r="F232" t="s">
-        <v>889</v>
+        <v>985</v>
       </c>
       <c r="G232" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="H232" s="4"/>
       <c r="I232" t="s">
@@ -10445,7 +10517,7 @@
         <v>621</v>
       </c>
       <c r="B233" t="s">
-        <v>1056</v>
+        <v>1052</v>
       </c>
       <c r="D233" t="s">
         <v>889</v>
@@ -10457,20 +10529,25 @@
         <v>889</v>
       </c>
       <c r="G233" t="s">
-        <v>1057</v>
+        <v>1053</v>
       </c>
       <c r="H233" s="4"/>
       <c r="I233" t="s">
-        <v>1042</v>
-      </c>
-      <c r="L233" s="7"/>
+        <v>233</v>
+      </c>
+      <c r="K233" s="6" t="s">
+        <v>899</v>
+      </c>
+      <c r="L233" s="7" t="s">
+        <v>900</v>
+      </c>
     </row>
     <row r="234" spans="1:12">
       <c r="A234" t="s">
         <v>621</v>
       </c>
       <c r="B234" t="s">
-        <v>1058</v>
+        <v>1054</v>
       </c>
       <c r="D234" t="s">
         <v>889</v>
@@ -10482,7 +10559,7 @@
         <v>889</v>
       </c>
       <c r="G234" t="s">
-        <v>1059</v>
+        <v>1055</v>
       </c>
       <c r="H234" s="4"/>
       <c r="I234" t="s">
@@ -10495,92 +10572,78 @@
         <v>621</v>
       </c>
       <c r="B235" t="s">
-        <v>45</v>
+        <v>1056</v>
       </c>
       <c r="D235" t="s">
-        <v>293</v>
+        <v>889</v>
       </c>
       <c r="E235" t="s">
-        <v>293</v>
+        <v>889</v>
       </c>
       <c r="F235" t="s">
-        <v>293</v>
+        <v>889</v>
       </c>
       <c r="G235" t="s">
-        <v>760</v>
-      </c>
-      <c r="H235" s="4" t="s">
-        <v>761</v>
-      </c>
+        <v>1057</v>
+      </c>
+      <c r="H235" s="4"/>
       <c r="I235" t="s">
-        <v>762</v>
-      </c>
-      <c r="J235" t="s">
-        <v>763</v>
-      </c>
-      <c r="L235" s="7" t="s">
-        <v>764</v>
-      </c>
+        <v>1042</v>
+      </c>
+      <c r="L235" s="7"/>
     </row>
     <row r="236" spans="1:12">
       <c r="A236" t="s">
         <v>621</v>
       </c>
       <c r="B236" t="s">
-        <v>1017</v>
+        <v>1058</v>
       </c>
       <c r="D236" t="s">
-        <v>1018</v>
+        <v>889</v>
       </c>
       <c r="E236" t="s">
-        <v>1018</v>
+        <v>889</v>
       </c>
       <c r="F236" t="s">
-        <v>1018</v>
+        <v>889</v>
       </c>
       <c r="G236" t="s">
-        <v>1019</v>
-      </c>
-      <c r="H236" s="4" t="s">
-        <v>761</v>
-      </c>
+        <v>1059</v>
+      </c>
+      <c r="H236" s="4"/>
       <c r="I236" t="s">
-        <v>1020</v>
-      </c>
-      <c r="J236" t="s">
-        <v>1021</v>
-      </c>
-      <c r="L236" s="7" t="s">
-        <v>764</v>
-      </c>
+        <v>1042</v>
+      </c>
+      <c r="L236" s="7"/>
     </row>
     <row r="237" spans="1:12">
       <c r="A237" t="s">
         <v>621</v>
       </c>
       <c r="B237" t="s">
-        <v>1024</v>
+        <v>45</v>
       </c>
       <c r="D237" t="s">
-        <v>1018</v>
+        <v>293</v>
       </c>
       <c r="E237" t="s">
-        <v>1018</v>
+        <v>293</v>
       </c>
       <c r="F237" t="s">
-        <v>1018</v>
+        <v>293</v>
       </c>
       <c r="G237" t="s">
-        <v>1025</v>
+        <v>760</v>
       </c>
       <c r="H237" s="4" t="s">
         <v>761</v>
       </c>
       <c r="I237" t="s">
-        <v>1027</v>
+        <v>762</v>
       </c>
       <c r="J237" t="s">
-        <v>1027</v>
+        <v>763</v>
       </c>
       <c r="L237" s="7" t="s">
         <v>764</v>
@@ -10591,34 +10654,31 @@
         <v>621</v>
       </c>
       <c r="B238" t="s">
-        <v>1060</v>
+        <v>1017</v>
       </c>
       <c r="D238" t="s">
-        <v>793</v>
+        <v>1018</v>
       </c>
       <c r="E238" t="s">
-        <v>793</v>
+        <v>1018</v>
       </c>
       <c r="F238" t="s">
-        <v>793</v>
+        <v>1018</v>
       </c>
       <c r="G238" t="s">
-        <v>1061</v>
+        <v>1019</v>
       </c>
       <c r="H238" s="4" t="s">
-        <v>1062</v>
+        <v>761</v>
       </c>
       <c r="I238" t="s">
-        <v>1063</v>
+        <v>1020</v>
       </c>
       <c r="J238" t="s">
-        <v>1063</v>
-      </c>
-      <c r="K238" t="s">
-        <v>1110</v>
+        <v>1021</v>
       </c>
       <c r="L238" s="7" t="s">
-        <v>1064</v>
+        <v>764</v>
       </c>
     </row>
     <row r="239" spans="1:12">
@@ -10626,34 +10686,31 @@
         <v>621</v>
       </c>
       <c r="B239" t="s">
-        <v>1065</v>
+        <v>1024</v>
       </c>
       <c r="D239" t="s">
-        <v>1066</v>
+        <v>1018</v>
       </c>
       <c r="E239" t="s">
-        <v>1066</v>
+        <v>1018</v>
       </c>
       <c r="F239" t="s">
-        <v>1066</v>
+        <v>1018</v>
       </c>
       <c r="G239" t="s">
-        <v>561</v>
+        <v>1025</v>
       </c>
       <c r="H239" s="4" t="s">
-        <v>562</v>
+        <v>761</v>
       </c>
       <c r="I239" t="s">
-        <v>563</v>
+        <v>1027</v>
       </c>
       <c r="J239" t="s">
-        <v>563</v>
-      </c>
-      <c r="K239" t="s">
-        <v>564</v>
+        <v>1027</v>
       </c>
       <c r="L239" s="7" t="s">
-        <v>565</v>
+        <v>764</v>
       </c>
     </row>
     <row r="240" spans="1:12">
@@ -10661,34 +10718,34 @@
         <v>621</v>
       </c>
       <c r="B240" t="s">
-        <v>1067</v>
+        <v>1060</v>
       </c>
       <c r="D240" t="s">
-        <v>1066</v>
+        <v>793</v>
       </c>
       <c r="E240" t="s">
-        <v>1066</v>
+        <v>793</v>
       </c>
       <c r="F240" t="s">
-        <v>1066</v>
+        <v>793</v>
       </c>
       <c r="G240" t="s">
-        <v>555</v>
+        <v>1061</v>
       </c>
       <c r="H240" s="4" t="s">
-        <v>761</v>
+        <v>1062</v>
       </c>
       <c r="I240" t="s">
-        <v>557</v>
+        <v>1063</v>
       </c>
       <c r="J240" t="s">
-        <v>557</v>
+        <v>1063</v>
       </c>
       <c r="K240" t="s">
-        <v>558</v>
+        <v>1110</v>
       </c>
       <c r="L240" s="7" t="s">
-        <v>559</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="241" spans="1:12">
@@ -10696,7 +10753,7 @@
         <v>621</v>
       </c>
       <c r="B241" t="s">
-        <v>1068</v>
+        <v>1065</v>
       </c>
       <c r="D241" t="s">
         <v>1066</v>
@@ -10707,37 +10764,58 @@
       <c r="F241" t="s">
         <v>1066</v>
       </c>
-      <c r="G241" s="10" t="s">
-        <v>1109</v>
-      </c>
-      <c r="H241" s="5"/>
-      <c r="I241" s="19"/>
-      <c r="J241" s="19"/>
-      <c r="K241" s="20"/>
-      <c r="L241" s="21"/>
+      <c r="G241" t="s">
+        <v>561</v>
+      </c>
+      <c r="H241" s="4" t="s">
+        <v>562</v>
+      </c>
+      <c r="I241" t="s">
+        <v>563</v>
+      </c>
+      <c r="J241" t="s">
+        <v>563</v>
+      </c>
+      <c r="K241" t="s">
+        <v>564</v>
+      </c>
+      <c r="L241" s="7" t="s">
+        <v>565</v>
+      </c>
     </row>
     <row r="242" spans="1:12">
       <c r="A242" t="s">
         <v>621</v>
       </c>
       <c r="B242" t="s">
-        <v>415</v>
+        <v>1067</v>
       </c>
       <c r="D242" t="s">
-        <v>625</v>
+        <v>1066</v>
       </c>
       <c r="E242" t="s">
-        <v>625</v>
+        <v>1066</v>
       </c>
       <c r="F242" t="s">
-        <v>625</v>
-      </c>
-      <c r="G242" s="10" t="s">
-        <v>1109</v>
-      </c>
-      <c r="H242" s="4"/>
+        <v>1066</v>
+      </c>
+      <c r="G242" t="s">
+        <v>555</v>
+      </c>
+      <c r="H242" s="4" t="s">
+        <v>761</v>
+      </c>
+      <c r="I242" t="s">
+        <v>557</v>
+      </c>
+      <c r="J242" t="s">
+        <v>557</v>
+      </c>
+      <c r="K242" t="s">
+        <v>558</v>
+      </c>
       <c r="L242" s="7" t="s">
-        <v>649</v>
+        <v>559</v>
       </c>
     </row>
     <row r="243" spans="1:12">
@@ -10745,39 +10823,32 @@
         <v>621</v>
       </c>
       <c r="B243" t="s">
-        <v>420</v>
+        <v>1068</v>
       </c>
       <c r="D243" t="s">
-        <v>625</v>
+        <v>1066</v>
       </c>
       <c r="E243" t="s">
-        <v>625</v>
+        <v>1066</v>
       </c>
       <c r="F243" t="s">
-        <v>657</v>
-      </c>
-      <c r="G243" t="s">
-        <v>1069</v>
-      </c>
-      <c r="H243" s="4" t="s">
-        <v>1070</v>
-      </c>
-      <c r="I243" t="s">
-        <v>1071</v>
-      </c>
-      <c r="K243" t="s">
-        <v>1111</v>
-      </c>
-      <c r="L243" s="7" t="s">
-        <v>1072</v>
-      </c>
+        <v>1066</v>
+      </c>
+      <c r="G243" s="10" t="s">
+        <v>1109</v>
+      </c>
+      <c r="H243" s="5"/>
+      <c r="I243" s="19"/>
+      <c r="J243" s="19"/>
+      <c r="K243" s="20"/>
+      <c r="L243" s="21"/>
     </row>
     <row r="244" spans="1:12">
       <c r="A244" t="s">
         <v>621</v>
       </c>
       <c r="B244" t="s">
-        <v>427</v>
+        <v>415</v>
       </c>
       <c r="D244" t="s">
         <v>625</v>
@@ -10786,22 +10857,14 @@
         <v>625</v>
       </c>
       <c r="F244" t="s">
-        <v>657</v>
-      </c>
-      <c r="G244" t="s">
-        <v>1073</v>
-      </c>
-      <c r="H244" s="4" t="s">
-        <v>1074</v>
-      </c>
-      <c r="I244" t="s">
-        <v>1075</v>
-      </c>
-      <c r="K244" t="s">
-        <v>1112</v>
-      </c>
+        <v>625</v>
+      </c>
+      <c r="G244" s="10" t="s">
+        <v>1109</v>
+      </c>
+      <c r="H244" s="4"/>
       <c r="L244" s="7" t="s">
-        <v>1072</v>
+        <v>649</v>
       </c>
     </row>
     <row r="245" spans="1:12">
@@ -10809,7 +10872,7 @@
         <v>621</v>
       </c>
       <c r="B245" t="s">
-        <v>433</v>
+        <v>420</v>
       </c>
       <c r="D245" t="s">
         <v>625</v>
@@ -10821,19 +10884,19 @@
         <v>657</v>
       </c>
       <c r="G245" t="s">
-        <v>1076</v>
+        <v>1069</v>
       </c>
       <c r="H245" s="4" t="s">
-        <v>1077</v>
+        <v>1070</v>
       </c>
       <c r="I245" t="s">
-        <v>1078</v>
+        <v>1071</v>
       </c>
       <c r="K245" t="s">
-        <v>1113</v>
+        <v>1111</v>
       </c>
       <c r="L245" s="7" t="s">
-        <v>1079</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="246" spans="1:12">
@@ -10841,7 +10904,7 @@
         <v>621</v>
       </c>
       <c r="B246" t="s">
-        <v>1080</v>
+        <v>427</v>
       </c>
       <c r="D246" t="s">
         <v>625</v>
@@ -10853,22 +10916,19 @@
         <v>657</v>
       </c>
       <c r="G246" t="s">
-        <v>1081</v>
+        <v>1073</v>
       </c>
       <c r="H246" s="4" t="s">
-        <v>1082</v>
+        <v>1074</v>
       </c>
       <c r="I246" t="s">
-        <v>1083</v>
-      </c>
-      <c r="J246" s="17" t="s">
-        <v>1115</v>
+        <v>1075</v>
       </c>
       <c r="K246" t="s">
-        <v>1114</v>
+        <v>1112</v>
       </c>
       <c r="L246" s="7" t="s">
-        <v>1084</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="247" spans="1:12">
@@ -10876,31 +10936,31 @@
         <v>621</v>
       </c>
       <c r="B247" t="s">
-        <v>1085</v>
+        <v>433</v>
       </c>
       <c r="D247" t="s">
-        <v>673</v>
+        <v>625</v>
       </c>
       <c r="E247" t="s">
-        <v>673</v>
+        <v>625</v>
       </c>
       <c r="F247" t="s">
-        <v>1086</v>
+        <v>657</v>
       </c>
       <c r="G247" t="s">
-        <v>701</v>
+        <v>1076</v>
       </c>
       <c r="H247" s="4" t="s">
-        <v>702</v>
+        <v>1077</v>
       </c>
       <c r="I247" t="s">
-        <v>703</v>
+        <v>1078</v>
       </c>
       <c r="K247" t="s">
-        <v>704</v>
+        <v>1113</v>
       </c>
       <c r="L247" s="7" t="s">
-        <v>665</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="248" spans="1:12">
@@ -10908,31 +10968,34 @@
         <v>621</v>
       </c>
       <c r="B248" t="s">
-        <v>1087</v>
+        <v>1080</v>
       </c>
       <c r="D248" t="s">
-        <v>673</v>
+        <v>625</v>
       </c>
       <c r="E248" t="s">
-        <v>673</v>
+        <v>625</v>
       </c>
       <c r="F248" t="s">
-        <v>674</v>
+        <v>657</v>
       </c>
       <c r="G248" t="s">
-        <v>709</v>
+        <v>1081</v>
       </c>
       <c r="H248" s="4" t="s">
-        <v>710</v>
+        <v>1082</v>
       </c>
       <c r="I248" t="s">
-        <v>711</v>
+        <v>1083</v>
+      </c>
+      <c r="J248" s="17" t="s">
+        <v>1115</v>
       </c>
       <c r="K248" t="s">
-        <v>712</v>
+        <v>1114</v>
       </c>
       <c r="L248" s="7" t="s">
-        <v>643</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="249" spans="1:12">
@@ -10940,7 +11003,7 @@
         <v>621</v>
       </c>
       <c r="B249" t="s">
-        <v>1088</v>
+        <v>1085</v>
       </c>
       <c r="D249" t="s">
         <v>673</v>
@@ -10949,25 +11012,22 @@
         <v>673</v>
       </c>
       <c r="F249" t="s">
-        <v>674</v>
+        <v>1086</v>
       </c>
       <c r="G249" t="s">
-        <v>691</v>
+        <v>701</v>
       </c>
       <c r="H249" s="4" t="s">
-        <v>692</v>
+        <v>702</v>
       </c>
       <c r="I249" t="s">
-        <v>693</v>
-      </c>
-      <c r="J249" t="s">
-        <v>694</v>
+        <v>703</v>
       </c>
       <c r="K249" t="s">
-        <v>695</v>
+        <v>704</v>
       </c>
       <c r="L249" s="7" t="s">
-        <v>683</v>
+        <v>665</v>
       </c>
     </row>
     <row r="250" spans="1:12">
@@ -10975,34 +11035,31 @@
         <v>621</v>
       </c>
       <c r="B250" t="s">
-        <v>1089</v>
+        <v>1087</v>
       </c>
       <c r="D250" t="s">
-        <v>719</v>
+        <v>673</v>
       </c>
       <c r="E250" t="s">
-        <v>719</v>
+        <v>673</v>
       </c>
       <c r="F250" t="s">
-        <v>719</v>
+        <v>674</v>
       </c>
       <c r="G250" t="s">
-        <v>1090</v>
+        <v>709</v>
       </c>
       <c r="H250" s="4" t="s">
-        <v>780</v>
+        <v>710</v>
       </c>
       <c r="I250" t="s">
-        <v>781</v>
-      </c>
-      <c r="J250" t="s">
-        <v>782</v>
+        <v>711</v>
       </c>
       <c r="K250" t="s">
-        <v>783</v>
+        <v>712</v>
       </c>
       <c r="L250" s="7" t="s">
-        <v>784</v>
+        <v>643</v>
       </c>
     </row>
     <row r="251" spans="1:12">
@@ -11010,45 +11067,152 @@
         <v>621</v>
       </c>
       <c r="B251" t="s">
+        <v>1088</v>
+      </c>
+      <c r="D251" t="s">
+        <v>673</v>
+      </c>
+      <c r="E251" t="s">
+        <v>673</v>
+      </c>
+      <c r="F251" t="s">
+        <v>674</v>
+      </c>
+      <c r="G251" t="s">
+        <v>691</v>
+      </c>
+      <c r="H251" s="4" t="s">
+        <v>692</v>
+      </c>
+      <c r="I251" t="s">
+        <v>693</v>
+      </c>
+      <c r="J251" t="s">
+        <v>694</v>
+      </c>
+      <c r="K251" t="s">
+        <v>695</v>
+      </c>
+      <c r="L251" s="7" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="252" spans="1:12">
+      <c r="A252" t="s">
+        <v>621</v>
+      </c>
+      <c r="B252" t="s">
+        <v>1089</v>
+      </c>
+      <c r="D252" t="s">
+        <v>719</v>
+      </c>
+      <c r="E252" t="s">
+        <v>719</v>
+      </c>
+      <c r="F252" t="s">
+        <v>719</v>
+      </c>
+      <c r="G252" t="s">
+        <v>1090</v>
+      </c>
+      <c r="H252" s="4" t="s">
+        <v>780</v>
+      </c>
+      <c r="I252" t="s">
+        <v>781</v>
+      </c>
+      <c r="J252" t="s">
+        <v>782</v>
+      </c>
+      <c r="K252" t="s">
+        <v>783</v>
+      </c>
+      <c r="L252" s="7" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="253" spans="1:12">
+      <c r="A253" t="s">
+        <v>621</v>
+      </c>
+      <c r="B253" t="s">
         <v>1091</v>
       </c>
-      <c r="D251" t="s">
+      <c r="D253" t="s">
         <v>719</v>
       </c>
-      <c r="E251" t="s">
+      <c r="E253" t="s">
         <v>719</v>
       </c>
-      <c r="F251" t="s">
+      <c r="F253" t="s">
         <v>720</v>
       </c>
-      <c r="G251" t="s">
+      <c r="G253" t="s">
         <v>743</v>
       </c>
-      <c r="H251" s="4" t="s">
+      <c r="H253" s="4" t="s">
         <v>744</v>
       </c>
-      <c r="I251" t="s">
+      <c r="I253" t="s">
         <v>745</v>
       </c>
-      <c r="J251" t="s">
+      <c r="J253" t="s">
         <v>746</v>
       </c>
-      <c r="K251" t="s">
+      <c r="K253" t="s">
         <v>747</v>
       </c>
-      <c r="L251" s="7" t="s">
+      <c r="L253" s="7" t="s">
         <v>748</v>
+      </c>
+    </row>
+    <row r="254" spans="1:12">
+      <c r="A254" t="s">
+        <v>621</v>
+      </c>
+      <c r="B254">
+        <v>199</v>
+      </c>
+      <c r="D254" t="s">
+        <v>1066</v>
+      </c>
+      <c r="E254" t="s">
+        <v>1066</v>
+      </c>
+      <c r="F254" t="s">
+        <v>1066</v>
+      </c>
+      <c r="G254" s="3" t="s">
+        <v>1131</v>
+      </c>
+      <c r="H254" s="3" t="s">
+        <v>1132</v>
+      </c>
+      <c r="I254" s="29" t="s">
+        <v>1133</v>
+      </c>
+      <c r="J254" s="29" t="s">
+        <v>1134</v>
+      </c>
+      <c r="K254" t="s">
+        <v>1135</v>
+      </c>
+      <c r="L254" t="s">
+        <v>1136</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="K157" r:id="rId1"/>
-    <hyperlink ref="K159" r:id="rId2"/>
-    <hyperlink ref="K155" r:id="rId3"/>
-    <hyperlink ref="K172" r:id="rId4"/>
-    <hyperlink ref="K165" r:id="rId5"/>
+    <hyperlink ref="K158" r:id="rId1"/>
+    <hyperlink ref="K160" r:id="rId2"/>
+    <hyperlink ref="K156" r:id="rId3"/>
+    <hyperlink ref="K173" r:id="rId4"/>
+    <hyperlink ref="K166" r:id="rId5"/>
+    <hyperlink ref="K176" r:id="rId6"/>
+    <hyperlink ref="K143" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>